<commit_message>
masters: regenereret fra plan.json
</commit_message>
<xml_diff>
--- a/data/Fast_as_Fifty_Masterplan_2026.xlsx
+++ b/data/Fast_as_Fifty_Masterplan_2026.xlsx
@@ -546,7 +546,7 @@
         </is>
       </c>
       <c r="B5" s="4" t="n">
-        <v>72.3</v>
+        <v>71.8</v>
       </c>
       <c r="C5" s="4" t="n">
         <v>68</v>
@@ -569,7 +569,7 @@
         </is>
       </c>
       <c r="B6" s="4" t="n">
-        <v>21.9</v>
+        <v>22.4</v>
       </c>
       <c r="C6" s="4" t="n">
         <v>16</v>
@@ -615,7 +615,7 @@
         </is>
       </c>
       <c r="B8" s="4" t="n">
-        <v>3.85</v>
+        <v>3.87</v>
       </c>
       <c r="C8" s="4" t="n">
         <v>4.71</v>
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>49.3</v>
+        <v>50.7</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>88</v>
@@ -3636,7 +3636,7 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-15</t>
+          <t>2026-06-16</t>
         </is>
       </c>
       <c r="B5" s="8" t="n"/>
@@ -3644,19 +3644,19 @@
       <c r="D5" s="8" t="n"/>
       <c r="E5" s="7" t="n"/>
       <c r="F5" s="8" t="n">
-        <v>-19.5</v>
+        <v>-26.4</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>8.9</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-16</t>
+          <t>2026-06-17</t>
         </is>
       </c>
       <c r="B6" s="8" t="n"/>
@@ -3664,19 +3664,19 @@
       <c r="D6" s="8" t="n"/>
       <c r="E6" s="7" t="n"/>
       <c r="F6" s="8" t="n">
-        <v>-26.4</v>
+        <v>-19.9</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>73</v>
+        <v>66</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>7.5</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-17</t>
+          <t>2026-06-18</t>
         </is>
       </c>
       <c r="B7" s="8" t="n"/>
@@ -3684,807 +3684,811 @@
       <c r="D7" s="8" t="n"/>
       <c r="E7" s="7" t="n"/>
       <c r="F7" s="8" t="n">
-        <v>-19.9</v>
+        <v>-15.3</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>66</v>
+        <v>82</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>9.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-18</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n"/>
-      <c r="C8" s="7" t="n"/>
-      <c r="D8" s="8" t="n"/>
-      <c r="E8" s="7" t="n"/>
+          <t>2026-06-19</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>73</v>
+      </c>
+      <c r="C8" s="7" t="n">
+        <v>73</v>
+      </c>
+      <c r="D8" s="8" t="n">
+        <v>21.7</v>
+      </c>
+      <c r="E8" s="7" t="n">
+        <v>21.7</v>
+      </c>
       <c r="F8" s="8" t="n">
-        <v>-15.3</v>
+        <v>-9.4</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>8</v>
+        <v>6.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-19</t>
+          <t>2026-06-20</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>73</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>73</v>
+        <v>73.2</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>21.7</v>
+        <v>22.4</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>21.7</v>
+        <v>22.05</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-9.4</v>
+        <v>-12</v>
       </c>
       <c r="G9" s="9" t="n">
-        <v>84</v>
+        <v>69</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>6.4</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-06-20</t>
+          <t>2026-06-21</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>73.40000000000001</v>
+        <v>73.59999999999999</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>73.2</v>
+        <v>73.33</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>22.4</v>
+        <v>21.7</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>22.05</v>
+        <v>21.93</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>-12</v>
+        <v>-12.4</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>69</v>
+        <v>60</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>8.800000000000001</v>
+        <v>5.6</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-06-21</t>
+          <t>2026-06-22</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
-        <v>73.59999999999999</v>
+        <v>73.2</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>73.33</v>
+        <v>73.3</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>21.93</v>
+        <v>21.9</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-12.4</v>
+        <v>-9.300000000000001</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>60</v>
+        <v>65</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>5.6</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-06-22</t>
+          <t>2026-06-23</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>73.2</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>73.3</v>
+        <v>73.31999999999999</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>21.8</v>
+        <v>22.4</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-9.300000000000001</v>
+        <v>-9.699999999999999</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>65</v>
+        <v>70</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>8.699999999999999</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-06-23</t>
+          <t>2026-06-24</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>73.40000000000001</v>
+        <v>72.5</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>73.31999999999999</v>
+        <v>73.18000000000001</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>22.4</v>
+        <v>23.1</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>22</v>
+        <v>22.18</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-9.699999999999999</v>
+        <v>-7.4</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>70</v>
+        <v>78</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>7.8</v>
+        <v>5.8</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-06-24</t>
+          <t>2026-06-25</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>72.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>73.18000000000001</v>
+        <v>73.14</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>23.1</v>
+        <v>22.7</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>22.18</v>
+        <v>22.26</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>-7.4</v>
+        <v>-11.1</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>78</v>
+        <v>58</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>5.8</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-06-25</t>
+          <t>2026-06-26</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>73.14</v>
+        <v>73.16</v>
       </c>
       <c r="D15" s="8" t="n">
         <v>22.7</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>22.26</v>
+        <v>22.4</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-11.1</v>
+        <v>-10.9</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>58</v>
+        <v>56</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>7.3</v>
+        <v>8</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>73.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>73.16</v>
+        <v>73.2</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>22.7</v>
+        <v>21.6</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>22.4</v>
+        <v>22.29</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>-10.9</v>
+        <v>-16</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B17" s="8" t="n">
-        <v>73.7</v>
+        <v>73.2</v>
       </c>
       <c r="C17" s="7" t="n">
-        <v>73.2</v>
+        <v>73.14</v>
       </c>
       <c r="D17" s="8" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="E17" s="7" t="n">
-        <v>22.29</v>
+        <v>22.3</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-16</v>
+        <v>-10.1</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>7.9</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>73.2</v>
+        <v>73.3</v>
       </c>
       <c r="C18" s="7" t="n">
-        <v>73.14</v>
+        <v>73.16</v>
       </c>
       <c r="D18" s="8" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="E18" s="7" t="n">
-        <v>22.3</v>
+        <v>22.31</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>-10.1</v>
+        <v>-5.9</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B19" s="8" t="n">
-        <v>73.3</v>
+        <v>72.8</v>
       </c>
       <c r="C19" s="7" t="n">
-        <v>73.16</v>
+        <v>73.06999999999999</v>
       </c>
       <c r="D19" s="8" t="n">
-        <v>21.9</v>
+        <v>23.2</v>
       </c>
       <c r="E19" s="7" t="n">
-        <v>22.31</v>
+        <v>22.43</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-5.9</v>
+        <v>-9.9</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B20" s="8" t="n">
         <v>72.8</v>
       </c>
       <c r="C20" s="7" t="n">
-        <v>73.06999999999999</v>
+        <v>73.11</v>
       </c>
       <c r="D20" s="8" t="n">
-        <v>23.2</v>
+        <v>23</v>
       </c>
       <c r="E20" s="7" t="n">
-        <v>22.43</v>
+        <v>22.41</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>-9.9</v>
+        <v>-13.3</v>
       </c>
       <c r="G20" s="9" t="n">
         <v>68</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>7.4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B21" s="8" t="n">
-        <v>72.8</v>
+        <v>72.5</v>
       </c>
       <c r="C21" s="7" t="n">
-        <v>73.11</v>
+        <v>73.06</v>
       </c>
       <c r="D21" s="8" t="n">
-        <v>23</v>
+        <v>21.7</v>
       </c>
       <c r="E21" s="7" t="n">
-        <v>22.41</v>
+        <v>22.27</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-13.3</v>
+        <v>-16.6</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
         <v>72.5</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>73.06</v>
+        <v>72.97</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>21.7</v>
+        <v>22.6</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>22.27</v>
+        <v>22.26</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>-16.6</v>
+        <v>-11.8</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>72.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>72.97</v>
+        <v>72.86</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>22.6</v>
+        <v>21.3</v>
       </c>
       <c r="E23" s="7" t="n">
-        <v>22.26</v>
+        <v>22.21</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-11.8</v>
+        <v>-21.1</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>72.86</v>
+        <v>72.8</v>
       </c>
       <c r="D24" s="8" t="n">
-        <v>21.3</v>
+        <v>22</v>
       </c>
       <c r="E24" s="7" t="n">
-        <v>22.21</v>
+        <v>22.24</v>
       </c>
       <c r="F24" s="8" t="n">
-        <v>-21.1</v>
+        <v>-25.6</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>6</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B25" s="8" t="n">
-        <v>72.8</v>
+        <v>72.5</v>
       </c>
       <c r="C25" s="7" t="n">
-        <v>72.8</v>
+        <v>72.69</v>
       </c>
       <c r="D25" s="8" t="n">
-        <v>22</v>
+        <v>21.5</v>
       </c>
       <c r="E25" s="7" t="n">
-        <v>22.24</v>
+        <v>22.19</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-25.6</v>
+        <v>-18.3</v>
       </c>
       <c r="G25" s="9" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>7.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B26" s="8" t="n">
-        <v>72.5</v>
+        <v>72.3</v>
       </c>
       <c r="C26" s="7" t="n">
-        <v>72.69</v>
+        <v>72.61</v>
       </c>
       <c r="D26" s="8" t="n">
-        <v>21.5</v>
+        <v>21.9</v>
       </c>
       <c r="E26" s="7" t="n">
-        <v>22.19</v>
+        <v>22</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>-18.3</v>
+        <v>-16</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>7.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B27" s="8" t="n">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C27" s="7" t="n">
-        <v>72.61</v>
+        <v>72.56</v>
       </c>
       <c r="D27" s="8" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="E27" s="7" t="n">
-        <v>22</v>
+        <v>21.83</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>-16</v>
+        <v>-10.4</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="B28" s="8" t="n">
-        <v>72.40000000000001</v>
-      </c>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B28" s="8" t="n"/>
       <c r="C28" s="7" t="n">
-        <v>72.56</v>
-      </c>
-      <c r="D28" s="8" t="n">
-        <v>21.8</v>
-      </c>
+        <v>72.56999999999999</v>
+      </c>
+      <c r="D28" s="8" t="n"/>
       <c r="E28" s="7" t="n">
-        <v>21.83</v>
+        <v>21.85</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>-10.4</v>
+        <v>-6.2</v>
       </c>
       <c r="G28" s="9" t="n">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B29" s="8" t="n"/>
       <c r="C29" s="7" t="n">
-        <v>72.56999999999999</v>
+        <v>72.58</v>
       </c>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="7" t="n">
-        <v>21.85</v>
+        <v>21.7</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-6.2</v>
+        <v>-12.3</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>7</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="7" t="n">
-        <v>72.58</v>
+        <v>72.5</v>
       </c>
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="7" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>-12.3</v>
+        <v>-6.6</v>
       </c>
       <c r="G30" s="9" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B31" s="8" t="n"/>
       <c r="C31" s="7" t="n">
-        <v>72.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D31" s="8" t="n"/>
       <c r="E31" s="7" t="n">
-        <v>21.8</v>
+        <v>21.73</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-6.6</v>
+        <v>-5.7</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B32" s="8" t="n"/>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B32" s="8" t="n">
+        <v>72.59999999999999</v>
+      </c>
       <c r="C32" s="7" t="n">
-        <v>72.40000000000001</v>
-      </c>
-      <c r="D32" s="8" t="n"/>
+        <v>72.43000000000001</v>
+      </c>
+      <c r="D32" s="8" t="n">
+        <v>21.2</v>
+      </c>
       <c r="E32" s="7" t="n">
-        <v>21.73</v>
+        <v>21.63</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>-5.7</v>
+        <v>-4.3</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>72.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>72.43000000000001</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>21.2</v>
+        <v>21.7</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>21.63</v>
+        <v>21.57</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-4.3</v>
+        <v>-7.5</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>72.2</v>
+        <v>71.7</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>72.17</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="E34" s="7" t="n">
         <v>21.57</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>-7.5</v>
+        <v>-10.9</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>71.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>72.17</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="D35" s="8" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E35" s="7" t="n">
         <v>21.8</v>
       </c>
-      <c r="E35" s="7" t="n">
-        <v>21.57</v>
-      </c>
       <c r="F35" s="8" t="n">
-        <v>-10.9</v>
+        <v>-7.7</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="B36" s="8" t="n">
-        <v>71.90000000000001</v>
-      </c>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B36" s="8" t="n"/>
       <c r="C36" s="7" t="n">
         <v>72.09999999999999</v>
       </c>
-      <c r="D36" s="8" t="n">
-        <v>22.5</v>
-      </c>
+      <c r="D36" s="8" t="n"/>
       <c r="E36" s="7" t="n">
         <v>21.8</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>-7.7</v>
+        <v>-8.9</v>
       </c>
       <c r="G36" s="9" t="n">
         <v>50</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B37" s="8" t="n"/>
@@ -4496,19 +4500,19 @@
         <v>21.8</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-8.9</v>
+        <v>-12.5</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="H37" s="10" t="n">
-        <v>7.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B38" s="8" t="n"/>
@@ -4520,274 +4524,278 @@
         <v>21.8</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>-12.5</v>
+        <v>-11.2</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>6.2</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B39" s="8" t="n"/>
       <c r="C39" s="7" t="n">
-        <v>72.09999999999999</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="D39" s="8" t="n"/>
       <c r="E39" s="7" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-11.2</v>
+        <v>-13.4</v>
       </c>
       <c r="G39" s="9" t="n">
         <v>63</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>8.800000000000001</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B40" s="8" t="n"/>
       <c r="C40" s="7" t="n">
-        <v>71.93000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="D40" s="8" t="n"/>
       <c r="E40" s="7" t="n">
-        <v>22</v>
+        <v>22.15</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>-13.4</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="G40" s="9" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="H40" s="10" t="n">
-        <v>6.7</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B41" s="8" t="n"/>
       <c r="C41" s="7" t="n">
-        <v>71.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="D41" s="8" t="n"/>
       <c r="E41" s="7" t="n">
-        <v>22.15</v>
+        <v>22.5</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-8.199999999999999</v>
+        <v>-12.4</v>
       </c>
       <c r="G41" s="9" t="n">
         <v>71</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>8.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="n"/>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>71.59999999999999</v>
+      </c>
       <c r="C42" s="7" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="D42" s="8" t="n"/>
+        <v>71.59999999999999</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>20.5</v>
+      </c>
       <c r="E42" s="7" t="n">
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>-12.4</v>
+        <v>-7.8</v>
       </c>
       <c r="G42" s="9" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H42" s="10" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>71.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>71.59999999999999</v>
+        <v>71.75</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>20.5</v>
+        <v>21.4</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>20.5</v>
+        <v>20.95</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-7.8</v>
+        <v>-3.1</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>7.4</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>71.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>71.75</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>20.95</v>
+        <v>21.13</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>-3.1</v>
+        <v>-11.8</v>
       </c>
       <c r="G44" s="9" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="H44" s="10" t="n">
-        <v>8.800000000000001</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>72.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>72.09999999999999</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>21.13</v>
+        <v>21.25</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-11.8</v>
+        <v>-9.6</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>6.8</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>72.40000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>72.18000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>21.25</v>
+        <v>21.22</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>-9.6</v>
+        <v>-8.6</v>
       </c>
       <c r="G46" s="9" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="H46" s="10" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>72.3</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>72.2</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="D47" s="8" t="n">
-        <v>21.1</v>
+        <v>21.9</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>21.22</v>
+        <v>21.33</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-8.6</v>
+        <v>-13.5</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>72.09999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>72.18000000000001</v>
+        <v>72.23</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>21.33</v>
+        <v>21.43</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>-13.5</v>
+        <v>-7.1</v>
       </c>
       <c r="G48" s="9" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H48" s="10" t="n">
         <v>7.7</v>
@@ -4796,510 +4804,510 @@
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B49" s="8" t="n">
-        <v>72.5</v>
+        <v>72.7</v>
       </c>
       <c r="C49" s="7" t="n">
-        <v>72.23</v>
+        <v>72.39</v>
       </c>
       <c r="D49" s="8" t="n">
         <v>22</v>
       </c>
       <c r="E49" s="7" t="n">
-        <v>21.43</v>
+        <v>21.64</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-7.1</v>
+        <v>-12.5</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B50" s="8" t="n">
-        <v>72.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C50" s="7" t="n">
         <v>72.39</v>
       </c>
       <c r="D50" s="8" t="n">
-        <v>22</v>
+        <v>21.7</v>
       </c>
       <c r="E50" s="7" t="n">
-        <v>21.64</v>
+        <v>21.69</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>-12.5</v>
+        <v>-6.8</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="H50" s="10" t="n">
-        <v>7.3</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B51" s="8" t="n">
-        <v>71.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C51" s="7" t="n">
-        <v>72.39</v>
+        <v>72.36</v>
       </c>
       <c r="D51" s="8" t="n">
-        <v>21.7</v>
+        <v>20.6</v>
       </c>
       <c r="E51" s="7" t="n">
-        <v>21.69</v>
+        <v>21.56</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-6.8</v>
+        <v>-0.2</v>
       </c>
       <c r="G51" s="9" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>8.300000000000001</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="B52" s="8" t="n">
-        <v>72.59999999999999</v>
-      </c>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B52" s="8" t="n"/>
       <c r="C52" s="7" t="n">
-        <v>72.36</v>
-      </c>
-      <c r="D52" s="8" t="n">
-        <v>20.6</v>
-      </c>
+        <v>72.34999999999999</v>
+      </c>
+      <c r="D52" s="8" t="n"/>
       <c r="E52" s="7" t="n">
-        <v>21.56</v>
+        <v>21.55</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>-0.2</v>
+        <v>-2.4</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="H52" s="10" t="n">
-        <v>6.9</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B53" s="8" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B53" s="8" t="n">
+        <v>72.90000000000001</v>
+      </c>
       <c r="C53" s="7" t="n">
-        <v>72.34999999999999</v>
-      </c>
-      <c r="D53" s="8" t="n"/>
+        <v>72.45</v>
+      </c>
+      <c r="D53" s="8" t="n">
+        <v>21.8</v>
+      </c>
       <c r="E53" s="7" t="n">
-        <v>21.55</v>
+        <v>21.67</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-2.4</v>
+        <v>-6</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>4.3</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B54" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="C54" s="7" t="n">
-        <v>72.45</v>
+        <v>72.47</v>
       </c>
       <c r="D54" s="8" t="n">
-        <v>21.8</v>
+        <v>21.1</v>
       </c>
       <c r="E54" s="7" t="n">
-        <v>21.67</v>
+        <v>21.53</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>-6</v>
+        <v>-4.5</v>
       </c>
       <c r="G54" s="9" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>7.9</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B55" s="8" t="n">
-        <v>72.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="C55" s="7" t="n">
-        <v>72.47</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D55" s="8" t="n">
-        <v>21.1</v>
+        <v>21.6</v>
       </c>
       <c r="E55" s="7" t="n">
-        <v>21.53</v>
+        <v>21.47</v>
       </c>
       <c r="F55" s="8" t="n">
-        <v>-4.5</v>
+        <v>-2.1</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H55" s="10" t="n">
-        <v>7.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B56" s="8" t="n">
-        <v>72.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C56" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>72.31999999999999</v>
       </c>
       <c r="D56" s="8" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="E56" s="7" t="n">
-        <v>21.47</v>
+        <v>21.43</v>
       </c>
       <c r="F56" s="8" t="n">
-        <v>-2.1</v>
+        <v>-4.1</v>
       </c>
       <c r="G56" s="9" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H56" s="10" t="n">
-        <v>9.300000000000001</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>72.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C57" s="7" t="n">
-        <v>72.31999999999999</v>
+        <v>72.23</v>
       </c>
       <c r="D57" s="8" t="n">
-        <v>21.8</v>
+        <v>21.5</v>
       </c>
       <c r="E57" s="7" t="n">
-        <v>21.43</v>
+        <v>21.4</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>-4.1</v>
+        <v>-1.6</v>
       </c>
       <c r="G57" s="9" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H57" s="10" t="n">
-        <v>7.7</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>71.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="C58" s="7" t="n">
-        <v>72.23</v>
+        <v>72.3</v>
       </c>
       <c r="D58" s="8" t="n">
         <v>21.5</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>21.4</v>
+        <v>21.55</v>
       </c>
       <c r="F58" s="8" t="n">
-        <v>-1.6</v>
+        <v>-15.1</v>
       </c>
       <c r="G58" s="9" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="H58" s="10" t="n">
-        <v>8.699999999999999</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>73</v>
+        <v>72.8</v>
       </c>
       <c r="C59" s="7" t="n">
-        <v>72.3</v>
+        <v>72.37</v>
       </c>
       <c r="D59" s="8" t="n">
-        <v>21.5</v>
+        <v>22.5</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>21.55</v>
+        <v>21.69</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>-15.1</v>
+        <v>-10.3</v>
       </c>
       <c r="G59" s="9" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="H59" s="10" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B60" s="8" t="n">
-        <v>72.8</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B60" s="8" t="n"/>
       <c r="C60" s="7" t="n">
-        <v>72.37</v>
-      </c>
-      <c r="D60" s="8" t="n">
-        <v>22.5</v>
-      </c>
+        <v>72.28</v>
+      </c>
+      <c r="D60" s="8" t="n"/>
       <c r="E60" s="7" t="n">
-        <v>21.69</v>
+        <v>21.67</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>-10.3</v>
+        <v>-14.8</v>
       </c>
       <c r="G60" s="9" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H60" s="10" t="n">
-        <v>5.7</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B61" s="8" t="n"/>
       <c r="C61" s="7" t="n">
-        <v>72.28</v>
+        <v>72.3</v>
       </c>
       <c r="D61" s="8" t="n"/>
       <c r="E61" s="7" t="n">
-        <v>21.67</v>
+        <v>21.78</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>-14.8</v>
+        <v>-15.7</v>
       </c>
       <c r="G61" s="9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H61" s="10" t="n">
-        <v>9.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B62" s="8" t="n"/>
       <c r="C62" s="7" t="n">
-        <v>72.3</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="D62" s="8" t="n"/>
       <c r="E62" s="7" t="n">
-        <v>21.78</v>
+        <v>21.82</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>-15.7</v>
+        <v>-15.4</v>
       </c>
       <c r="G62" s="9" t="n">
         <v>60</v>
       </c>
       <c r="H62" s="10" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B63" s="8" t="n"/>
       <c r="C63" s="7" t="n">
-        <v>72.34999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D63" s="8" t="n"/>
       <c r="E63" s="7" t="n">
-        <v>21.82</v>
+        <v>21.83</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>-15.4</v>
+        <v>-8.9</v>
       </c>
       <c r="G63" s="9" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="H63" s="10" t="n">
-        <v>7.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B64" s="8" t="n"/>
       <c r="C64" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="D64" s="8" t="n"/>
       <c r="E64" s="7" t="n">
-        <v>21.83</v>
+        <v>22</v>
       </c>
       <c r="F64" s="8" t="n">
-        <v>-8.9</v>
+        <v>-6.7</v>
       </c>
       <c r="G64" s="9" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H64" s="10" t="n">
-        <v>6.2</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B65" s="8" t="n"/>
       <c r="C65" s="7" t="n">
-        <v>72.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="D65" s="8" t="n"/>
       <c r="E65" s="7" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="F65" s="8" t="n">
-        <v>-6.7</v>
+        <v>-4.8</v>
       </c>
       <c r="G65" s="9" t="n">
         <v>47</v>
       </c>
       <c r="H65" s="10" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B66" s="8" t="n"/>
-      <c r="C66" s="7" t="n">
-        <v>72.8</v>
-      </c>
+      <c r="C66" s="7" t="n"/>
       <c r="D66" s="8" t="n"/>
-      <c r="E66" s="7" t="n">
-        <v>22.5</v>
-      </c>
+      <c r="E66" s="7" t="n"/>
       <c r="F66" s="8" t="n">
-        <v>-4.8</v>
+        <v>0.6</v>
       </c>
       <c r="G66" s="9" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="H66" s="10" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="B67" s="8" t="n"/>
-      <c r="C67" s="7" t="n"/>
-      <c r="D67" s="8" t="n"/>
-      <c r="E67" s="7" t="n"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B67" s="8" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="C67" s="7" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="D67" s="8" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E67" s="7" t="n">
+        <v>21.9</v>
+      </c>
       <c r="F67" s="8" t="n">
-        <v>0.6</v>
+        <v>3.5</v>
       </c>
       <c r="G67" s="9" t="n">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="H67" s="10" t="n">
-        <v>6.3</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>73.2</v>
+        <v>72.8</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>73.2</v>
+        <v>73</v>
       </c>
       <c r="D68" s="8" t="n">
         <v>21.9</v>
@@ -5308,395 +5316,395 @@
         <v>21.9</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>3.5</v>
+        <v>-9.4</v>
       </c>
       <c r="G68" s="9" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="H68" s="10" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B69" s="8" t="n">
-        <v>72.8</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="C69" s="7" t="n">
-        <v>73</v>
+        <v>72.97</v>
       </c>
       <c r="D69" s="8" t="n">
-        <v>21.9</v>
+        <v>21.3</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>21.9</v>
+        <v>21.7</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>-9.4</v>
+        <v>-6.9</v>
       </c>
       <c r="G69" s="9" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="H69" s="10" t="n">
-        <v>8.300000000000001</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>72.97</v>
+        <v>72.88</v>
       </c>
       <c r="D70" s="8" t="n">
-        <v>21.3</v>
+        <v>20.9</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>-6.9</v>
+        <v>-3.2</v>
       </c>
       <c r="G70" s="9" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H70" s="10" t="n">
-        <v>9.6</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>72.59999999999999</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C71" s="7" t="n">
-        <v>72.88</v>
+        <v>73.08</v>
       </c>
       <c r="D71" s="8" t="n">
         <v>20.9</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>21.5</v>
+        <v>21.38</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>-3.2</v>
+        <v>0.9</v>
       </c>
       <c r="G71" s="9" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H71" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>73.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>73.08</v>
+        <v>73</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>20.9</v>
+        <v>21.8</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>21.38</v>
+        <v>21.45</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>0.9</v>
+        <v>2.7</v>
       </c>
       <c r="G72" s="9" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H72" s="10" t="n">
-        <v>6.8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B73" s="8" t="n">
-        <v>72.59999999999999</v>
-      </c>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B73" s="8" t="n"/>
       <c r="C73" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="D73" s="8" t="n">
-        <v>21.8</v>
-      </c>
+      <c r="D73" s="8" t="n"/>
       <c r="E73" s="7" t="n">
         <v>21.45</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="G73" s="9" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="H73" s="10" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="n"/>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="n">
+        <v>71.90000000000001</v>
+      </c>
       <c r="C74" s="7" t="n">
-        <v>73</v>
-      </c>
-      <c r="D74" s="8" t="n"/>
+        <v>72.78</v>
+      </c>
+      <c r="D74" s="8" t="n">
+        <v>20.7</v>
+      </c>
       <c r="E74" s="7" t="n">
-        <v>21.45</v>
+        <v>21.25</v>
       </c>
       <c r="F74" s="8" t="n">
-        <v>2.4</v>
+        <v>4</v>
       </c>
       <c r="G74" s="9" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H74" s="10" t="n">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B75" s="8" t="n">
-        <v>71.90000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="C75" s="7" t="n">
-        <v>72.78</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="D75" s="8" t="n">
-        <v>20.7</v>
+        <v>21.6</v>
       </c>
       <c r="E75" s="7" t="n">
-        <v>21.25</v>
+        <v>21.2</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>4</v>
+        <v>-3.6</v>
       </c>
       <c r="G75" s="9" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="H75" s="10" t="n">
-        <v>6.7</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B76" s="8" t="n">
-        <v>71.5</v>
+        <v>71</v>
       </c>
       <c r="C76" s="7" t="n">
-        <v>72.56999999999999</v>
+        <v>72.25</v>
       </c>
       <c r="D76" s="8" t="n">
-        <v>21.6</v>
+        <v>21.9</v>
       </c>
       <c r="E76" s="7" t="n">
-        <v>21.2</v>
+        <v>21.3</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>-3.6</v>
+        <v>1</v>
       </c>
       <c r="G76" s="9" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H76" s="10" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B77" s="8" t="n">
-        <v>71</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="C77" s="7" t="n">
-        <v>72.25</v>
+        <v>72.08</v>
       </c>
       <c r="D77" s="8" t="n">
-        <v>21.9</v>
+        <v>21.4</v>
       </c>
       <c r="E77" s="7" t="n">
-        <v>21.3</v>
+        <v>21.38</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>1</v>
+        <v>5.9</v>
       </c>
       <c r="G77" s="9" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="H77" s="10" t="n">
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B78" s="8" t="n">
-        <v>71.59999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="C78" s="7" t="n">
-        <v>72.08</v>
+        <v>71.81999999999999</v>
       </c>
       <c r="D78" s="8" t="n">
-        <v>21.4</v>
+        <v>20.8</v>
       </c>
       <c r="E78" s="7" t="n">
-        <v>21.38</v>
+        <v>21.37</v>
       </c>
       <c r="F78" s="8" t="n">
-        <v>5.9</v>
+        <v>9.5</v>
       </c>
       <c r="G78" s="9" t="n">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="H78" s="10" t="n">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B79" s="8" t="n">
-        <v>72.3</v>
+        <v>72.5</v>
       </c>
       <c r="C79" s="7" t="n">
-        <v>71.81999999999999</v>
+        <v>71.8</v>
       </c>
       <c r="D79" s="8" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="E79" s="7" t="n">
-        <v>21.37</v>
+        <v>21.33</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="G79" s="9" t="n">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="H79" s="10" t="n">
-        <v>8.4</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B80" s="8" t="n">
-        <v>72.5</v>
+        <v>73</v>
       </c>
       <c r="C80" s="7" t="n">
-        <v>71.8</v>
+        <v>71.97</v>
       </c>
       <c r="D80" s="8" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="E80" s="7" t="n">
-        <v>21.33</v>
+        <v>21.44</v>
       </c>
       <c r="F80" s="8" t="n">
-        <v>6</v>
+        <v>2.7</v>
       </c>
       <c r="G80" s="9" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H80" s="10" t="n">
-        <v>7.5</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>73</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>71.97</v>
+        <v>72.14</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>22.1</v>
+        <v>22.6</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>21.44</v>
+        <v>21.71</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>2.7</v>
+        <v>6.1</v>
       </c>
       <c r="G81" s="9" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="H81" s="10" t="n">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B82" s="8" t="n">
-        <v>73.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C82" s="7" t="n">
-        <v>72.14</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="D82" s="8" t="n">
-        <v>22.6</v>
+        <v>20.8</v>
       </c>
       <c r="E82" s="7" t="n">
-        <v>21.71</v>
+        <v>21.6</v>
       </c>
       <c r="F82" s="8" t="n">
-        <v>6.1</v>
+        <v>4.8</v>
       </c>
       <c r="G82" s="9" t="n">
         <v>63</v>
@@ -5708,187 +5716,183 @@
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B83" s="8" t="n">
-        <v>72.2</v>
+        <v>72.3</v>
       </c>
       <c r="C83" s="7" t="n">
-        <v>72.23999999999999</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="D83" s="8" t="n">
-        <v>20.8</v>
+        <v>21.3</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>21.6</v>
+        <v>21.51</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="G83" s="9" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="H83" s="10" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B84" s="8" t="n">
         <v>72.3</v>
       </c>
       <c r="C84" s="7" t="n">
-        <v>72.43000000000001</v>
+        <v>72.53</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>21.3</v>
+        <v>21.9</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>21.51</v>
+        <v>21.59</v>
       </c>
       <c r="F84" s="8" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G84" s="9" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="H84" s="10" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="B85" s="8" t="n">
-        <v>72.3</v>
-      </c>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B85" s="8" t="n"/>
       <c r="C85" s="7" t="n">
-        <v>72.53</v>
-      </c>
-      <c r="D85" s="8" t="n">
-        <v>21.9</v>
-      </c>
+        <v>72.56999999999999</v>
+      </c>
+      <c r="D85" s="8" t="n"/>
       <c r="E85" s="7" t="n">
-        <v>21.59</v>
+        <v>21.72</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>5.3</v>
+        <v>7.7</v>
       </c>
       <c r="G85" s="9" t="n">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="H85" s="10" t="n">
-        <v>8.9</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B86" s="8" t="n"/>
       <c r="C86" s="7" t="n">
-        <v>72.56999999999999</v>
+        <v>72.58</v>
       </c>
       <c r="D86" s="8" t="n"/>
       <c r="E86" s="7" t="n">
-        <v>21.72</v>
+        <v>21.74</v>
       </c>
       <c r="F86" s="8" t="n">
-        <v>7.7</v>
+        <v>-7.3</v>
       </c>
       <c r="G86" s="9" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H86" s="10" t="n">
-        <v>6.6</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B87" s="8" t="n"/>
       <c r="C87" s="7" t="n">
-        <v>72.58</v>
+        <v>72.48</v>
       </c>
       <c r="D87" s="8" t="n"/>
       <c r="E87" s="7" t="n">
-        <v>21.74</v>
+        <v>21.65</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>-7.3</v>
+        <v>-2.2</v>
       </c>
       <c r="G87" s="9" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="H87" s="10" t="n">
-        <v>4.1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B88" s="8" t="n"/>
       <c r="C88" s="7" t="n">
-        <v>72.48</v>
+        <v>72.27</v>
       </c>
       <c r="D88" s="8" t="n"/>
       <c r="E88" s="7" t="n">
-        <v>21.65</v>
+        <v>21.33</v>
       </c>
       <c r="F88" s="8" t="n">
-        <v>-2.2</v>
+        <v>1.7</v>
       </c>
       <c r="G88" s="9" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H88" s="10" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B89" s="8" t="n"/>
       <c r="C89" s="7" t="n">
-        <v>72.27</v>
+        <v>72.3</v>
       </c>
       <c r="D89" s="8" t="n"/>
       <c r="E89" s="7" t="n">
-        <v>21.33</v>
+        <v>21.6</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>1.7</v>
+        <v>5</v>
       </c>
       <c r="G89" s="9" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H89" s="10" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B90" s="8" t="n"/>
@@ -5897,124 +5901,128 @@
       </c>
       <c r="D90" s="8" t="n"/>
       <c r="E90" s="7" t="n">
-        <v>21.6</v>
+        <v>21.9</v>
       </c>
       <c r="F90" s="8" t="n">
-        <v>5</v>
+        <v>1.9</v>
       </c>
       <c r="G90" s="9" t="n">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="H90" s="10" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B91" s="8" t="n"/>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B91" s="8" t="n">
+        <v>73.7</v>
+      </c>
       <c r="C91" s="7" t="n">
-        <v>72.3</v>
-      </c>
-      <c r="D91" s="8" t="n"/>
+        <v>73.7</v>
+      </c>
+      <c r="D91" s="8" t="n">
+        <v>20.9</v>
+      </c>
       <c r="E91" s="7" t="n">
-        <v>21.9</v>
+        <v>20.9</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="G91" s="9" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H91" s="10" t="n">
-        <v>7.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>73.7</v>
+        <v>72.5</v>
       </c>
       <c r="C92" s="7" t="n">
-        <v>73.7</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="D92" s="8" t="n">
-        <v>20.9</v>
+        <v>21.4</v>
       </c>
       <c r="E92" s="7" t="n">
-        <v>20.9</v>
+        <v>21.15</v>
       </c>
       <c r="F92" s="8" t="n">
-        <v>2.2</v>
+        <v>5.9</v>
       </c>
       <c r="G92" s="9" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="H92" s="10" t="n">
-        <v>6.7</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>72.5</v>
+        <v>72.3</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>73.09999999999999</v>
+        <v>72.83</v>
       </c>
       <c r="D93" s="8" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E93" s="7" t="n">
         <v>21.4</v>
       </c>
-      <c r="E93" s="7" t="n">
-        <v>21.15</v>
-      </c>
       <c r="F93" s="8" t="n">
-        <v>5.9</v>
+        <v>4</v>
       </c>
       <c r="G93" s="9" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H93" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B94" s="8" t="n">
-        <v>72.3</v>
+        <v>71.8</v>
       </c>
       <c r="C94" s="7" t="n">
-        <v>72.83</v>
+        <v>72.58</v>
       </c>
       <c r="D94" s="8" t="n">
-        <v>21.9</v>
+        <v>22.4</v>
       </c>
       <c r="E94" s="7" t="n">
-        <v>21.4</v>
+        <v>21.65</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>1</v>
+        <v>-6.1</v>
       </c>
       <c r="G94" s="9" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="H94" s="10" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
   </sheetData>
@@ -6115,16 +6123,16 @@
         <v>47</v>
       </c>
       <c r="E5" s="8" t="n">
-        <v>49.3</v>
+        <v>50.7</v>
       </c>
       <c r="F5" s="4" t="n">
         <v>150</v>
       </c>
       <c r="G5" s="4" t="n">
-        <v>221</v>
+        <v>289</v>
       </c>
       <c r="H5" s="11" t="n">
-        <v>71</v>
+        <v>139</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
QA 24/9: ugemetadata og tests efter flyt af styrke/svøm/FTP-test (#19)
* QA 24/9: ugemetadata og tests efter flyt af styrke/svøm/FTP-test

* masters: regenereret fra plan.json

---------

Co-authored-by: github-actions[bot] <41898282+github-actions[bot]@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/data/Fast_as_Fifty_Masterplan_2026.xlsx
+++ b/data/Fast_as_Fifty_Masterplan_2026.xlsx
@@ -638,7 +638,7 @@
         </is>
       </c>
       <c r="B9" s="4" t="n">
-        <v>48.5</v>
+        <v>48.7</v>
       </c>
       <c r="C9" s="4" t="n">
         <v>88</v>
@@ -1629,7 +1629,7 @@
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>Cut starter. FTP-test tor 24/9. Styrke Functional 4 A/B 2×/uge. Svøm 1×/uge (ons/fre) genindført 11/9 — må ikke koste cykeltid.</t>
+          <t>Cut starter. FTP-test flyttet 24/9 til tor 8/10 (træt uge). Fra uge 41: styrke man+lør 45 min, svøm fre (ons alternativ).</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>Recovery. Ingen test.</t>
+          <t>Recovery. FTP-test tor 8/10 efter Mallorca.</t>
         </is>
       </c>
     </row>
@@ -3636,579 +3636,575 @@
     <row r="5">
       <c r="A5" s="4" t="inlineStr">
         <is>
-          <t>2026-06-26</t>
+          <t>2026-06-27</t>
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>73.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="C5" s="7" t="n">
-        <v>73.09999999999999</v>
+        <v>73.7</v>
       </c>
       <c r="D5" s="8" t="n">
-        <v>22.7</v>
+        <v>21.6</v>
       </c>
       <c r="E5" s="7" t="n">
-        <v>22.7</v>
+        <v>21.6</v>
       </c>
       <c r="F5" s="8" t="n">
-        <v>-10.9</v>
+        <v>-16</v>
       </c>
       <c r="G5" s="9" t="n">
-        <v>56</v>
+        <v>60</v>
       </c>
       <c r="H5" s="10" t="n">
-        <v>8</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="inlineStr">
         <is>
-          <t>2026-06-27</t>
+          <t>2026-06-28</t>
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>73.7</v>
+        <v>73.2</v>
       </c>
       <c r="C6" s="7" t="n">
-        <v>73.40000000000001</v>
+        <v>73.45</v>
       </c>
       <c r="D6" s="8" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="E6" s="7" t="n">
-        <v>22.15</v>
+        <v>21.7</v>
       </c>
       <c r="F6" s="8" t="n">
-        <v>-16</v>
+        <v>-10.1</v>
       </c>
       <c r="G6" s="9" t="n">
-        <v>60</v>
+        <v>74</v>
       </c>
       <c r="H6" s="10" t="n">
-        <v>7.9</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="inlineStr">
         <is>
-          <t>2026-06-28</t>
+          <t>2026-06-29</t>
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>73.2</v>
+        <v>73.3</v>
       </c>
       <c r="C7" s="7" t="n">
-        <v>73.33</v>
+        <v>73.40000000000001</v>
       </c>
       <c r="D7" s="8" t="n">
-        <v>21.8</v>
+        <v>21.9</v>
       </c>
       <c r="E7" s="7" t="n">
-        <v>22.03</v>
+        <v>21.77</v>
       </c>
       <c r="F7" s="8" t="n">
-        <v>-10.1</v>
+        <v>-5.9</v>
       </c>
       <c r="G7" s="9" t="n">
-        <v>74</v>
+        <v>56</v>
       </c>
       <c r="H7" s="10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-06-30</t>
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>73.3</v>
+        <v>72.8</v>
       </c>
       <c r="C8" s="7" t="n">
-        <v>73.33</v>
+        <v>73.25</v>
       </c>
       <c r="D8" s="8" t="n">
-        <v>21.9</v>
+        <v>23.2</v>
       </c>
       <c r="E8" s="7" t="n">
-        <v>22</v>
+        <v>22.13</v>
       </c>
       <c r="F8" s="8" t="n">
-        <v>-5.9</v>
+        <v>-9.9</v>
       </c>
       <c r="G8" s="9" t="n">
-        <v>56</v>
+        <v>68</v>
       </c>
       <c r="H8" s="10" t="n">
-        <v>7.2</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="4" t="inlineStr">
         <is>
-          <t>2026-06-30</t>
+          <t>2026-07-01</t>
         </is>
       </c>
       <c r="B9" s="8" t="n">
         <v>72.8</v>
       </c>
       <c r="C9" s="7" t="n">
-        <v>73.22</v>
+        <v>73.16</v>
       </c>
       <c r="D9" s="8" t="n">
-        <v>23.2</v>
+        <v>23</v>
       </c>
       <c r="E9" s="7" t="n">
-        <v>22.24</v>
+        <v>22.3</v>
       </c>
       <c r="F9" s="8" t="n">
-        <v>-9.9</v>
+        <v>-13.3</v>
       </c>
       <c r="G9" s="9" t="n">
         <v>68</v>
       </c>
       <c r="H9" s="10" t="n">
-        <v>7.4</v>
+        <v>9</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="4" t="inlineStr">
         <is>
-          <t>2026-07-01</t>
+          <t>2026-07-02</t>
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>72.8</v>
+        <v>72.5</v>
       </c>
       <c r="C10" s="7" t="n">
-        <v>73.15000000000001</v>
+        <v>73.05</v>
       </c>
       <c r="D10" s="8" t="n">
-        <v>23</v>
+        <v>21.7</v>
       </c>
       <c r="E10" s="7" t="n">
-        <v>22.37</v>
+        <v>22.2</v>
       </c>
       <c r="F10" s="8" t="n">
-        <v>-13.3</v>
+        <v>-16.6</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>68</v>
+        <v>50</v>
       </c>
       <c r="H10" s="10" t="n">
-        <v>9</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" s="4" t="inlineStr">
         <is>
-          <t>2026-07-02</t>
+          <t>2026-07-03</t>
         </is>
       </c>
       <c r="B11" s="8" t="n">
         <v>72.5</v>
       </c>
       <c r="C11" s="7" t="n">
-        <v>73.06</v>
+        <v>72.97</v>
       </c>
       <c r="D11" s="8" t="n">
-        <v>21.7</v>
+        <v>22.6</v>
       </c>
       <c r="E11" s="7" t="n">
-        <v>22.27</v>
+        <v>22.26</v>
       </c>
       <c r="F11" s="8" t="n">
-        <v>-16.6</v>
+        <v>-11.8</v>
       </c>
       <c r="G11" s="9" t="n">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="H11" s="10" t="n">
-        <v>6.2</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="4" t="inlineStr">
         <is>
-          <t>2026-07-03</t>
+          <t>2026-07-04</t>
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>72.5</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="C12" s="7" t="n">
-        <v>72.97</v>
+        <v>72.86</v>
       </c>
       <c r="D12" s="8" t="n">
-        <v>22.6</v>
+        <v>21.3</v>
       </c>
       <c r="E12" s="7" t="n">
-        <v>22.26</v>
+        <v>22.21</v>
       </c>
       <c r="F12" s="8" t="n">
-        <v>-11.8</v>
+        <v>-21.1</v>
       </c>
       <c r="G12" s="9" t="n">
-        <v>52</v>
+        <v>39</v>
       </c>
       <c r="H12" s="10" t="n">
-        <v>6.6</v>
+        <v>6</v>
       </c>
     </row>
     <row r="13">
       <c r="A13" s="4" t="inlineStr">
         <is>
-          <t>2026-07-04</t>
+          <t>2026-07-05</t>
         </is>
       </c>
       <c r="B13" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="C13" s="7" t="n">
-        <v>72.86</v>
+        <v>72.8</v>
       </c>
       <c r="D13" s="8" t="n">
-        <v>21.3</v>
+        <v>22</v>
       </c>
       <c r="E13" s="7" t="n">
-        <v>22.21</v>
+        <v>22.24</v>
       </c>
       <c r="F13" s="8" t="n">
-        <v>-21.1</v>
+        <v>-25.6</v>
       </c>
       <c r="G13" s="9" t="n">
-        <v>39</v>
+        <v>56</v>
       </c>
       <c r="H13" s="10" t="n">
-        <v>6</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="4" t="inlineStr">
         <is>
-          <t>2026-07-05</t>
+          <t>2026-07-06</t>
         </is>
       </c>
       <c r="B14" s="8" t="n">
-        <v>72.8</v>
+        <v>72.5</v>
       </c>
       <c r="C14" s="7" t="n">
-        <v>72.8</v>
+        <v>72.69</v>
       </c>
       <c r="D14" s="8" t="n">
-        <v>22</v>
+        <v>21.5</v>
       </c>
       <c r="E14" s="7" t="n">
-        <v>22.24</v>
+        <v>22.19</v>
       </c>
       <c r="F14" s="8" t="n">
-        <v>-25.6</v>
+        <v>-18.3</v>
       </c>
       <c r="G14" s="9" t="n">
-        <v>56</v>
+        <v>67</v>
       </c>
       <c r="H14" s="10" t="n">
-        <v>7.6</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="4" t="inlineStr">
         <is>
-          <t>2026-07-06</t>
+          <t>2026-07-07</t>
         </is>
       </c>
       <c r="B15" s="8" t="n">
-        <v>72.5</v>
+        <v>72.3</v>
       </c>
       <c r="C15" s="7" t="n">
-        <v>72.69</v>
+        <v>72.61</v>
       </c>
       <c r="D15" s="8" t="n">
-        <v>21.5</v>
+        <v>21.9</v>
       </c>
       <c r="E15" s="7" t="n">
-        <v>22.19</v>
+        <v>22</v>
       </c>
       <c r="F15" s="8" t="n">
-        <v>-18.3</v>
+        <v>-16</v>
       </c>
       <c r="G15" s="9" t="n">
-        <v>67</v>
+        <v>71</v>
       </c>
       <c r="H15" s="10" t="n">
-        <v>7.1</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="4" t="inlineStr">
         <is>
-          <t>2026-07-07</t>
+          <t>2026-07-08</t>
         </is>
       </c>
       <c r="B16" s="8" t="n">
-        <v>72.3</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C16" s="7" t="n">
-        <v>72.61</v>
+        <v>72.56</v>
       </c>
       <c r="D16" s="8" t="n">
-        <v>21.9</v>
+        <v>21.8</v>
       </c>
       <c r="E16" s="7" t="n">
-        <v>22</v>
+        <v>21.83</v>
       </c>
       <c r="F16" s="8" t="n">
-        <v>-16</v>
+        <v>-10.4</v>
       </c>
       <c r="G16" s="9" t="n">
-        <v>71</v>
+        <v>66</v>
       </c>
       <c r="H16" s="10" t="n">
-        <v>8.9</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="4" t="inlineStr">
         <is>
-          <t>2026-07-08</t>
-        </is>
-      </c>
-      <c r="B17" s="8" t="n">
-        <v>72.40000000000001</v>
-      </c>
+          <t>2026-07-09</t>
+        </is>
+      </c>
+      <c r="B17" s="8" t="n"/>
       <c r="C17" s="7" t="n">
-        <v>72.56</v>
-      </c>
-      <c r="D17" s="8" t="n">
-        <v>21.8</v>
-      </c>
+        <v>72.56999999999999</v>
+      </c>
+      <c r="D17" s="8" t="n"/>
       <c r="E17" s="7" t="n">
-        <v>21.83</v>
+        <v>21.85</v>
       </c>
       <c r="F17" s="8" t="n">
-        <v>-10.4</v>
+        <v>-6.2</v>
       </c>
       <c r="G17" s="9" t="n">
-        <v>66</v>
+        <v>38</v>
       </c>
       <c r="H17" s="10" t="n">
-        <v>6.9</v>
+        <v>7</v>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="4" t="inlineStr">
         <is>
-          <t>2026-07-09</t>
+          <t>2026-07-10</t>
         </is>
       </c>
       <c r="B18" s="8" t="n"/>
       <c r="C18" s="7" t="n">
-        <v>72.56999999999999</v>
+        <v>72.58</v>
       </c>
       <c r="D18" s="8" t="n"/>
       <c r="E18" s="7" t="n">
-        <v>21.85</v>
+        <v>21.7</v>
       </c>
       <c r="F18" s="8" t="n">
-        <v>-6.2</v>
+        <v>-12.3</v>
       </c>
       <c r="G18" s="9" t="n">
-        <v>38</v>
+        <v>75</v>
       </c>
       <c r="H18" s="10" t="n">
-        <v>7</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="19">
       <c r="A19" s="4" t="inlineStr">
         <is>
-          <t>2026-07-10</t>
+          <t>2026-07-11</t>
         </is>
       </c>
       <c r="B19" s="8" t="n"/>
       <c r="C19" s="7" t="n">
-        <v>72.58</v>
+        <v>72.5</v>
       </c>
       <c r="D19" s="8" t="n"/>
       <c r="E19" s="7" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="F19" s="8" t="n">
-        <v>-12.3</v>
+        <v>-6.6</v>
       </c>
       <c r="G19" s="9" t="n">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="H19" s="10" t="n">
-        <v>8.4</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="4" t="inlineStr">
         <is>
-          <t>2026-07-11</t>
+          <t>2026-07-12</t>
         </is>
       </c>
       <c r="B20" s="8" t="n"/>
       <c r="C20" s="7" t="n">
-        <v>72.5</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D20" s="8" t="n"/>
       <c r="E20" s="7" t="n">
-        <v>21.8</v>
+        <v>21.73</v>
       </c>
       <c r="F20" s="8" t="n">
-        <v>-6.6</v>
+        <v>-5.7</v>
       </c>
       <c r="G20" s="9" t="n">
-        <v>76</v>
+        <v>53</v>
       </c>
       <c r="H20" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="4" t="inlineStr">
         <is>
-          <t>2026-07-12</t>
-        </is>
-      </c>
-      <c r="B21" s="8" t="n"/>
+          <t>2026-07-13</t>
+        </is>
+      </c>
+      <c r="B21" s="8" t="n">
+        <v>72.59999999999999</v>
+      </c>
       <c r="C21" s="7" t="n">
-        <v>72.40000000000001</v>
-      </c>
-      <c r="D21" s="8" t="n"/>
+        <v>72.43000000000001</v>
+      </c>
+      <c r="D21" s="8" t="n">
+        <v>21.2</v>
+      </c>
       <c r="E21" s="7" t="n">
-        <v>21.73</v>
+        <v>21.63</v>
       </c>
       <c r="F21" s="8" t="n">
-        <v>-5.7</v>
+        <v>-4.3</v>
       </c>
       <c r="G21" s="9" t="n">
-        <v>53</v>
+        <v>51</v>
       </c>
       <c r="H21" s="10" t="n">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="4" t="inlineStr">
         <is>
-          <t>2026-07-13</t>
+          <t>2026-07-14</t>
         </is>
       </c>
       <c r="B22" s="8" t="n">
-        <v>72.59999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C22" s="7" t="n">
-        <v>72.43000000000001</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D22" s="8" t="n">
-        <v>21.2</v>
+        <v>21.7</v>
       </c>
       <c r="E22" s="7" t="n">
-        <v>21.63</v>
+        <v>21.57</v>
       </c>
       <c r="F22" s="8" t="n">
-        <v>-4.3</v>
+        <v>-7.5</v>
       </c>
       <c r="G22" s="9" t="n">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="H22" s="10" t="n">
-        <v>7.2</v>
+        <v>7</v>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="4" t="inlineStr">
         <is>
-          <t>2026-07-14</t>
+          <t>2026-07-15</t>
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>72.2</v>
+        <v>71.7</v>
       </c>
       <c r="C23" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>72.17</v>
       </c>
       <c r="D23" s="8" t="n">
-        <v>21.7</v>
+        <v>21.8</v>
       </c>
       <c r="E23" s="7" t="n">
         <v>21.57</v>
       </c>
       <c r="F23" s="8" t="n">
-        <v>-7.5</v>
+        <v>-10.9</v>
       </c>
       <c r="G23" s="9" t="n">
-        <v>52</v>
+        <v>45</v>
       </c>
       <c r="H23" s="10" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="4" t="inlineStr">
         <is>
-          <t>2026-07-15</t>
+          <t>2026-07-16</t>
         </is>
       </c>
       <c r="B24" s="8" t="n">
-        <v>71.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C24" s="7" t="n">
-        <v>72.17</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="D24" s="8" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="E24" s="7" t="n">
         <v>21.8</v>
       </c>
-      <c r="E24" s="7" t="n">
-        <v>21.57</v>
-      </c>
       <c r="F24" s="8" t="n">
-        <v>-10.9</v>
+        <v>-7.7</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H24" s="10" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
     </row>
     <row r="25">
       <c r="A25" s="4" t="inlineStr">
         <is>
-          <t>2026-07-16</t>
-        </is>
-      </c>
-      <c r="B25" s="8" t="n">
-        <v>71.90000000000001</v>
-      </c>
+          <t>2026-07-17</t>
+        </is>
+      </c>
+      <c r="B25" s="8" t="n"/>
       <c r="C25" s="7" t="n">
         <v>72.09999999999999</v>
       </c>
-      <c r="D25" s="8" t="n">
-        <v>22.5</v>
-      </c>
+      <c r="D25" s="8" t="n"/>
       <c r="E25" s="7" t="n">
         <v>21.8</v>
       </c>
       <c r="F25" s="8" t="n">
-        <v>-7.7</v>
+        <v>-8.9</v>
       </c>
       <c r="G25" s="9" t="n">
         <v>50</v>
       </c>
       <c r="H25" s="10" t="n">
-        <v>6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="26">
       <c r="A26" s="4" t="inlineStr">
         <is>
-          <t>2026-07-17</t>
+          <t>2026-07-18</t>
         </is>
       </c>
       <c r="B26" s="8" t="n"/>
@@ -4220,19 +4216,19 @@
         <v>21.8</v>
       </c>
       <c r="F26" s="8" t="n">
-        <v>-8.9</v>
+        <v>-12.5</v>
       </c>
       <c r="G26" s="9" t="n">
-        <v>50</v>
+        <v>35</v>
       </c>
       <c r="H26" s="10" t="n">
-        <v>7.7</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="27">
       <c r="A27" s="4" t="inlineStr">
         <is>
-          <t>2026-07-18</t>
+          <t>2026-07-19</t>
         </is>
       </c>
       <c r="B27" s="8" t="n"/>
@@ -4244,274 +4240,278 @@
         <v>21.8</v>
       </c>
       <c r="F27" s="8" t="n">
-        <v>-12.5</v>
+        <v>-11.2</v>
       </c>
       <c r="G27" s="9" t="n">
-        <v>35</v>
+        <v>63</v>
       </c>
       <c r="H27" s="10" t="n">
-        <v>6.2</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="4" t="inlineStr">
         <is>
-          <t>2026-07-19</t>
+          <t>2026-07-20</t>
         </is>
       </c>
       <c r="B28" s="8" t="n"/>
       <c r="C28" s="7" t="n">
-        <v>72.09999999999999</v>
+        <v>71.93000000000001</v>
       </c>
       <c r="D28" s="8" t="n"/>
       <c r="E28" s="7" t="n">
-        <v>21.8</v>
+        <v>22</v>
       </c>
       <c r="F28" s="8" t="n">
-        <v>-11.2</v>
+        <v>-13.4</v>
       </c>
       <c r="G28" s="9" t="n">
         <v>63</v>
       </c>
       <c r="H28" s="10" t="n">
-        <v>8.800000000000001</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="4" t="inlineStr">
         <is>
-          <t>2026-07-20</t>
+          <t>2026-07-21</t>
         </is>
       </c>
       <c r="B29" s="8" t="n"/>
       <c r="C29" s="7" t="n">
-        <v>71.93000000000001</v>
+        <v>71.8</v>
       </c>
       <c r="D29" s="8" t="n"/>
       <c r="E29" s="7" t="n">
-        <v>22</v>
+        <v>22.15</v>
       </c>
       <c r="F29" s="8" t="n">
-        <v>-13.4</v>
+        <v>-8.199999999999999</v>
       </c>
       <c r="G29" s="9" t="n">
-        <v>63</v>
+        <v>71</v>
       </c>
       <c r="H29" s="10" t="n">
-        <v>6.7</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="4" t="inlineStr">
         <is>
-          <t>2026-07-21</t>
+          <t>2026-07-22</t>
         </is>
       </c>
       <c r="B30" s="8" t="n"/>
       <c r="C30" s="7" t="n">
-        <v>71.8</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="D30" s="8" t="n"/>
       <c r="E30" s="7" t="n">
-        <v>22.15</v>
+        <v>22.5</v>
       </c>
       <c r="F30" s="8" t="n">
-        <v>-8.199999999999999</v>
+        <v>-12.4</v>
       </c>
       <c r="G30" s="9" t="n">
         <v>71</v>
       </c>
       <c r="H30" s="10" t="n">
-        <v>8.4</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="31">
       <c r="A31" s="4" t="inlineStr">
         <is>
-          <t>2026-07-22</t>
-        </is>
-      </c>
-      <c r="B31" s="8" t="n"/>
+          <t>2026-07-23</t>
+        </is>
+      </c>
+      <c r="B31" s="8" t="n">
+        <v>71.59999999999999</v>
+      </c>
       <c r="C31" s="7" t="n">
-        <v>71.90000000000001</v>
-      </c>
-      <c r="D31" s="8" t="n"/>
+        <v>71.59999999999999</v>
+      </c>
+      <c r="D31" s="8" t="n">
+        <v>20.5</v>
+      </c>
       <c r="E31" s="7" t="n">
-        <v>22.5</v>
+        <v>20.5</v>
       </c>
       <c r="F31" s="8" t="n">
-        <v>-12.4</v>
+        <v>-7.8</v>
       </c>
       <c r="G31" s="9" t="n">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="H31" s="10" t="n">
-        <v>7.1</v>
+        <v>7.4</v>
       </c>
     </row>
     <row r="32">
       <c r="A32" s="4" t="inlineStr">
         <is>
-          <t>2026-07-23</t>
+          <t>2026-07-24</t>
         </is>
       </c>
       <c r="B32" s="8" t="n">
-        <v>71.59999999999999</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C32" s="7" t="n">
-        <v>71.59999999999999</v>
+        <v>71.75</v>
       </c>
       <c r="D32" s="8" t="n">
-        <v>20.5</v>
+        <v>21.4</v>
       </c>
       <c r="E32" s="7" t="n">
-        <v>20.5</v>
+        <v>20.95</v>
       </c>
       <c r="F32" s="8" t="n">
-        <v>-7.8</v>
+        <v>-3.1</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>70</v>
+        <v>74</v>
       </c>
       <c r="H32" s="10" t="n">
-        <v>7.4</v>
+        <v>8.800000000000001</v>
       </c>
     </row>
     <row r="33">
       <c r="A33" s="4" t="inlineStr">
         <is>
-          <t>2026-07-24</t>
+          <t>2026-07-25</t>
         </is>
       </c>
       <c r="B33" s="8" t="n">
-        <v>71.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="C33" s="7" t="n">
-        <v>71.75</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="D33" s="8" t="n">
-        <v>21.4</v>
+        <v>21.5</v>
       </c>
       <c r="E33" s="7" t="n">
-        <v>20.95</v>
+        <v>21.13</v>
       </c>
       <c r="F33" s="8" t="n">
-        <v>-3.1</v>
+        <v>-11.8</v>
       </c>
       <c r="G33" s="9" t="n">
-        <v>74</v>
+        <v>65</v>
       </c>
       <c r="H33" s="10" t="n">
-        <v>8.800000000000001</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="34">
       <c r="A34" s="4" t="inlineStr">
         <is>
-          <t>2026-07-25</t>
+          <t>2026-07-26</t>
         </is>
       </c>
       <c r="B34" s="8" t="n">
-        <v>72.8</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="C34" s="7" t="n">
-        <v>72.09999999999999</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="D34" s="8" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="E34" s="7" t="n">
-        <v>21.13</v>
+        <v>21.25</v>
       </c>
       <c r="F34" s="8" t="n">
-        <v>-11.8</v>
+        <v>-9.6</v>
       </c>
       <c r="G34" s="9" t="n">
-        <v>65</v>
+        <v>46</v>
       </c>
       <c r="H34" s="10" t="n">
-        <v>6.8</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="4" t="inlineStr">
         <is>
-          <t>2026-07-26</t>
+          <t>2026-07-27</t>
         </is>
       </c>
       <c r="B35" s="8" t="n">
-        <v>72.40000000000001</v>
+        <v>72.3</v>
       </c>
       <c r="C35" s="7" t="n">
-        <v>72.18000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="D35" s="8" t="n">
-        <v>21.6</v>
+        <v>21.1</v>
       </c>
       <c r="E35" s="7" t="n">
-        <v>21.25</v>
+        <v>21.22</v>
       </c>
       <c r="F35" s="8" t="n">
-        <v>-9.6</v>
+        <v>-8.6</v>
       </c>
       <c r="G35" s="9" t="n">
-        <v>46</v>
+        <v>60</v>
       </c>
       <c r="H35" s="10" t="n">
-        <v>8.6</v>
+        <v>9.199999999999999</v>
       </c>
     </row>
     <row r="36">
       <c r="A36" s="4" t="inlineStr">
         <is>
-          <t>2026-07-27</t>
+          <t>2026-07-28</t>
         </is>
       </c>
       <c r="B36" s="8" t="n">
-        <v>72.3</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="C36" s="7" t="n">
-        <v>72.2</v>
+        <v>72.18000000000001</v>
       </c>
       <c r="D36" s="8" t="n">
-        <v>21.1</v>
+        <v>21.9</v>
       </c>
       <c r="E36" s="7" t="n">
-        <v>21.22</v>
+        <v>21.33</v>
       </c>
       <c r="F36" s="8" t="n">
-        <v>-8.6</v>
+        <v>-13.5</v>
       </c>
       <c r="G36" s="9" t="n">
-        <v>60</v>
+        <v>66</v>
       </c>
       <c r="H36" s="10" t="n">
-        <v>9.199999999999999</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="4" t="inlineStr">
         <is>
-          <t>2026-07-28</t>
+          <t>2026-07-29</t>
         </is>
       </c>
       <c r="B37" s="8" t="n">
-        <v>72.09999999999999</v>
+        <v>72.5</v>
       </c>
       <c r="C37" s="7" t="n">
-        <v>72.18000000000001</v>
+        <v>72.23</v>
       </c>
       <c r="D37" s="8" t="n">
-        <v>21.9</v>
+        <v>22</v>
       </c>
       <c r="E37" s="7" t="n">
-        <v>21.33</v>
+        <v>21.43</v>
       </c>
       <c r="F37" s="8" t="n">
-        <v>-13.5</v>
+        <v>-7.1</v>
       </c>
       <c r="G37" s="9" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H37" s="10" t="n">
         <v>7.7</v>
@@ -4520,510 +4520,510 @@
     <row r="38">
       <c r="A38" s="4" t="inlineStr">
         <is>
-          <t>2026-07-29</t>
+          <t>2026-07-30</t>
         </is>
       </c>
       <c r="B38" s="8" t="n">
-        <v>72.5</v>
+        <v>72.7</v>
       </c>
       <c r="C38" s="7" t="n">
-        <v>72.23</v>
+        <v>72.39</v>
       </c>
       <c r="D38" s="8" t="n">
         <v>22</v>
       </c>
       <c r="E38" s="7" t="n">
-        <v>21.43</v>
+        <v>21.64</v>
       </c>
       <c r="F38" s="8" t="n">
-        <v>-7.1</v>
+        <v>-12.5</v>
       </c>
       <c r="G38" s="9" t="n">
-        <v>55</v>
+        <v>70</v>
       </c>
       <c r="H38" s="10" t="n">
-        <v>7.7</v>
+        <v>7.3</v>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="4" t="inlineStr">
         <is>
-          <t>2026-07-30</t>
+          <t>2026-07-31</t>
         </is>
       </c>
       <c r="B39" s="8" t="n">
-        <v>72.7</v>
+        <v>71.90000000000001</v>
       </c>
       <c r="C39" s="7" t="n">
         <v>72.39</v>
       </c>
       <c r="D39" s="8" t="n">
-        <v>22</v>
+        <v>21.7</v>
       </c>
       <c r="E39" s="7" t="n">
-        <v>21.64</v>
+        <v>21.69</v>
       </c>
       <c r="F39" s="8" t="n">
-        <v>-12.5</v>
+        <v>-6.8</v>
       </c>
       <c r="G39" s="9" t="n">
-        <v>70</v>
+        <v>47</v>
       </c>
       <c r="H39" s="10" t="n">
-        <v>7.3</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="4" t="inlineStr">
         <is>
-          <t>2026-07-31</t>
+          <t>2026-08-01</t>
         </is>
       </c>
       <c r="B40" s="8" t="n">
-        <v>71.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C40" s="7" t="n">
-        <v>72.39</v>
+        <v>72.36</v>
       </c>
       <c r="D40" s="8" t="n">
-        <v>21.7</v>
+        <v>20.6</v>
       </c>
       <c r="E40" s="7" t="n">
-        <v>21.69</v>
+        <v>21.56</v>
       </c>
       <c r="F40" s="8" t="n">
-        <v>-6.8</v>
+        <v>-0.2</v>
       </c>
       <c r="G40" s="9" t="n">
-        <v>47</v>
+        <v>23</v>
       </c>
       <c r="H40" s="10" t="n">
-        <v>8.300000000000001</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="4" t="inlineStr">
         <is>
-          <t>2026-08-01</t>
-        </is>
-      </c>
-      <c r="B41" s="8" t="n">
-        <v>72.59999999999999</v>
-      </c>
+          <t>2026-08-02</t>
+        </is>
+      </c>
+      <c r="B41" s="8" t="n"/>
       <c r="C41" s="7" t="n">
-        <v>72.36</v>
-      </c>
-      <c r="D41" s="8" t="n">
-        <v>20.6</v>
-      </c>
+        <v>72.34999999999999</v>
+      </c>
+      <c r="D41" s="8" t="n"/>
       <c r="E41" s="7" t="n">
-        <v>21.56</v>
+        <v>21.55</v>
       </c>
       <c r="F41" s="8" t="n">
-        <v>-0.2</v>
+        <v>-2.4</v>
       </c>
       <c r="G41" s="9" t="n">
-        <v>23</v>
+        <v>32</v>
       </c>
       <c r="H41" s="10" t="n">
-        <v>6.9</v>
+        <v>4.3</v>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="4" t="inlineStr">
         <is>
-          <t>2026-08-02</t>
-        </is>
-      </c>
-      <c r="B42" s="8" t="n"/>
+          <t>2026-08-03</t>
+        </is>
+      </c>
+      <c r="B42" s="8" t="n">
+        <v>72.90000000000001</v>
+      </c>
       <c r="C42" s="7" t="n">
-        <v>72.34999999999999</v>
-      </c>
-      <c r="D42" s="8" t="n"/>
+        <v>72.45</v>
+      </c>
+      <c r="D42" s="8" t="n">
+        <v>21.8</v>
+      </c>
       <c r="E42" s="7" t="n">
-        <v>21.55</v>
+        <v>21.67</v>
       </c>
       <c r="F42" s="8" t="n">
-        <v>-2.4</v>
+        <v>-6</v>
       </c>
       <c r="G42" s="9" t="n">
-        <v>32</v>
+        <v>54</v>
       </c>
       <c r="H42" s="10" t="n">
-        <v>4.3</v>
+        <v>7.9</v>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="4" t="inlineStr">
         <is>
-          <t>2026-08-03</t>
+          <t>2026-08-04</t>
         </is>
       </c>
       <c r="B43" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>72.2</v>
       </c>
       <c r="C43" s="7" t="n">
-        <v>72.45</v>
+        <v>72.47</v>
       </c>
       <c r="D43" s="8" t="n">
-        <v>21.8</v>
+        <v>21.1</v>
       </c>
       <c r="E43" s="7" t="n">
-        <v>21.67</v>
+        <v>21.53</v>
       </c>
       <c r="F43" s="8" t="n">
-        <v>-6</v>
+        <v>-4.5</v>
       </c>
       <c r="G43" s="9" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H43" s="10" t="n">
-        <v>7.9</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="4" t="inlineStr">
         <is>
-          <t>2026-08-04</t>
+          <t>2026-08-05</t>
         </is>
       </c>
       <c r="B44" s="8" t="n">
-        <v>72.2</v>
+        <v>72.09999999999999</v>
       </c>
       <c r="C44" s="7" t="n">
-        <v>72.47</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D44" s="8" t="n">
-        <v>21.1</v>
+        <v>21.6</v>
       </c>
       <c r="E44" s="7" t="n">
-        <v>21.53</v>
+        <v>21.47</v>
       </c>
       <c r="F44" s="8" t="n">
-        <v>-4.5</v>
+        <v>-2.1</v>
       </c>
       <c r="G44" s="9" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H44" s="10" t="n">
-        <v>7.1</v>
+        <v>9.300000000000001</v>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="4" t="inlineStr">
         <is>
-          <t>2026-08-05</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B45" s="8" t="n">
-        <v>72.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C45" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>72.31999999999999</v>
       </c>
       <c r="D45" s="8" t="n">
-        <v>21.6</v>
+        <v>21.8</v>
       </c>
       <c r="E45" s="7" t="n">
-        <v>21.47</v>
+        <v>21.43</v>
       </c>
       <c r="F45" s="8" t="n">
-        <v>-2.1</v>
+        <v>-4.1</v>
       </c>
       <c r="G45" s="9" t="n">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="H45" s="10" t="n">
-        <v>9.300000000000001</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="4" t="inlineStr">
         <is>
-          <t>2026-08-06</t>
+          <t>2026-08-07</t>
         </is>
       </c>
       <c r="B46" s="8" t="n">
-        <v>72.2</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C46" s="7" t="n">
-        <v>72.31999999999999</v>
+        <v>72.23</v>
       </c>
       <c r="D46" s="8" t="n">
-        <v>21.8</v>
+        <v>21.5</v>
       </c>
       <c r="E46" s="7" t="n">
-        <v>21.43</v>
+        <v>21.4</v>
       </c>
       <c r="F46" s="8" t="n">
-        <v>-4.1</v>
+        <v>-1.6</v>
       </c>
       <c r="G46" s="9" t="n">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H46" s="10" t="n">
-        <v>7.7</v>
+        <v>8.699999999999999</v>
       </c>
     </row>
     <row r="47">
       <c r="A47" s="4" t="inlineStr">
         <is>
-          <t>2026-08-07</t>
+          <t>2026-08-08</t>
         </is>
       </c>
       <c r="B47" s="8" t="n">
-        <v>71.40000000000001</v>
+        <v>73</v>
       </c>
       <c r="C47" s="7" t="n">
-        <v>72.23</v>
+        <v>72.3</v>
       </c>
       <c r="D47" s="8" t="n">
         <v>21.5</v>
       </c>
       <c r="E47" s="7" t="n">
-        <v>21.4</v>
+        <v>21.55</v>
       </c>
       <c r="F47" s="8" t="n">
-        <v>-1.6</v>
+        <v>-15.1</v>
       </c>
       <c r="G47" s="9" t="n">
-        <v>49</v>
+        <v>36</v>
       </c>
       <c r="H47" s="10" t="n">
-        <v>8.699999999999999</v>
+        <v>5.3</v>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="4" t="inlineStr">
         <is>
-          <t>2026-08-08</t>
+          <t>2026-08-09</t>
         </is>
       </c>
       <c r="B48" s="8" t="n">
-        <v>73</v>
+        <v>72.8</v>
       </c>
       <c r="C48" s="7" t="n">
-        <v>72.3</v>
+        <v>72.37</v>
       </c>
       <c r="D48" s="8" t="n">
-        <v>21.5</v>
+        <v>22.5</v>
       </c>
       <c r="E48" s="7" t="n">
-        <v>21.55</v>
+        <v>21.69</v>
       </c>
       <c r="F48" s="8" t="n">
-        <v>-15.1</v>
+        <v>-10.3</v>
       </c>
       <c r="G48" s="9" t="n">
-        <v>36</v>
+        <v>45</v>
       </c>
       <c r="H48" s="10" t="n">
-        <v>5.3</v>
+        <v>5.7</v>
       </c>
     </row>
     <row r="49">
       <c r="A49" s="4" t="inlineStr">
         <is>
-          <t>2026-08-09</t>
-        </is>
-      </c>
-      <c r="B49" s="8" t="n">
-        <v>72.8</v>
-      </c>
+          <t>2026-08-10</t>
+        </is>
+      </c>
+      <c r="B49" s="8" t="n"/>
       <c r="C49" s="7" t="n">
-        <v>72.37</v>
-      </c>
-      <c r="D49" s="8" t="n">
-        <v>22.5</v>
-      </c>
+        <v>72.28</v>
+      </c>
+      <c r="D49" s="8" t="n"/>
       <c r="E49" s="7" t="n">
-        <v>21.69</v>
+        <v>21.67</v>
       </c>
       <c r="F49" s="8" t="n">
-        <v>-10.3</v>
+        <v>-14.8</v>
       </c>
       <c r="G49" s="9" t="n">
-        <v>45</v>
+        <v>50</v>
       </c>
       <c r="H49" s="10" t="n">
-        <v>5.7</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="4" t="inlineStr">
         <is>
-          <t>2026-08-10</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="B50" s="8" t="n"/>
       <c r="C50" s="7" t="n">
-        <v>72.28</v>
+        <v>72.3</v>
       </c>
       <c r="D50" s="8" t="n"/>
       <c r="E50" s="7" t="n">
-        <v>21.67</v>
+        <v>21.78</v>
       </c>
       <c r="F50" s="8" t="n">
-        <v>-14.8</v>
+        <v>-15.7</v>
       </c>
       <c r="G50" s="9" t="n">
-        <v>50</v>
+        <v>60</v>
       </c>
       <c r="H50" s="10" t="n">
-        <v>9.1</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="4" t="inlineStr">
         <is>
-          <t>2026-08-11</t>
+          <t>2026-08-12</t>
         </is>
       </c>
       <c r="B51" s="8" t="n"/>
       <c r="C51" s="7" t="n">
-        <v>72.3</v>
+        <v>72.34999999999999</v>
       </c>
       <c r="D51" s="8" t="n"/>
       <c r="E51" s="7" t="n">
-        <v>21.78</v>
+        <v>21.82</v>
       </c>
       <c r="F51" s="8" t="n">
-        <v>-15.7</v>
+        <v>-15.4</v>
       </c>
       <c r="G51" s="9" t="n">
         <v>60</v>
       </c>
       <c r="H51" s="10" t="n">
-        <v>7.5</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="4" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-13</t>
         </is>
       </c>
       <c r="B52" s="8" t="n"/>
       <c r="C52" s="7" t="n">
-        <v>72.34999999999999</v>
+        <v>72.40000000000001</v>
       </c>
       <c r="D52" s="8" t="n"/>
       <c r="E52" s="7" t="n">
-        <v>21.82</v>
+        <v>21.83</v>
       </c>
       <c r="F52" s="8" t="n">
-        <v>-15.4</v>
+        <v>-8.9</v>
       </c>
       <c r="G52" s="9" t="n">
-        <v>60</v>
+        <v>52</v>
       </c>
       <c r="H52" s="10" t="n">
-        <v>7.8</v>
+        <v>6.2</v>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="4" t="inlineStr">
         <is>
-          <t>2026-08-13</t>
+          <t>2026-08-14</t>
         </is>
       </c>
       <c r="B53" s="8" t="n"/>
       <c r="C53" s="7" t="n">
-        <v>72.40000000000001</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="D53" s="8" t="n"/>
       <c r="E53" s="7" t="n">
-        <v>21.83</v>
+        <v>22</v>
       </c>
       <c r="F53" s="8" t="n">
-        <v>-8.9</v>
+        <v>-6.7</v>
       </c>
       <c r="G53" s="9" t="n">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="H53" s="10" t="n">
-        <v>6.2</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="4" t="inlineStr">
         <is>
-          <t>2026-08-14</t>
+          <t>2026-08-15</t>
         </is>
       </c>
       <c r="B54" s="8" t="n"/>
       <c r="C54" s="7" t="n">
-        <v>72.90000000000001</v>
+        <v>72.8</v>
       </c>
       <c r="D54" s="8" t="n"/>
       <c r="E54" s="7" t="n">
-        <v>22</v>
+        <v>22.5</v>
       </c>
       <c r="F54" s="8" t="n">
-        <v>-6.7</v>
+        <v>-4.8</v>
       </c>
       <c r="G54" s="9" t="n">
         <v>47</v>
       </c>
       <c r="H54" s="10" t="n">
-        <v>6.8</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="4" t="inlineStr">
         <is>
-          <t>2026-08-15</t>
+          <t>2026-08-16</t>
         </is>
       </c>
       <c r="B55" s="8" t="n"/>
-      <c r="C55" s="7" t="n">
-        <v>72.8</v>
-      </c>
+      <c r="C55" s="7" t="n"/>
       <c r="D55" s="8" t="n"/>
-      <c r="E55" s="7" t="n">
-        <v>22.5</v>
-      </c>
+      <c r="E55" s="7" t="n"/>
       <c r="F55" s="8" t="n">
-        <v>-4.8</v>
+        <v>0.6</v>
       </c>
       <c r="G55" s="9" t="n">
-        <v>47</v>
+        <v>56</v>
       </c>
       <c r="H55" s="10" t="n">
-        <v>7.2</v>
+        <v>6.3</v>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="4" t="inlineStr">
         <is>
-          <t>2026-08-16</t>
-        </is>
-      </c>
-      <c r="B56" s="8" t="n"/>
-      <c r="C56" s="7" t="n"/>
-      <c r="D56" s="8" t="n"/>
-      <c r="E56" s="7" t="n"/>
+          <t>2026-08-17</t>
+        </is>
+      </c>
+      <c r="B56" s="8" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="C56" s="7" t="n">
+        <v>73.2</v>
+      </c>
+      <c r="D56" s="8" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E56" s="7" t="n">
+        <v>21.9</v>
+      </c>
       <c r="F56" s="8" t="n">
-        <v>0.6</v>
+        <v>3.5</v>
       </c>
       <c r="G56" s="9" t="n">
-        <v>56</v>
+        <v>79</v>
       </c>
       <c r="H56" s="10" t="n">
-        <v>6.3</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="4" t="inlineStr">
         <is>
-          <t>2026-08-17</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B57" s="8" t="n">
-        <v>73.2</v>
+        <v>72.8</v>
       </c>
       <c r="C57" s="7" t="n">
-        <v>73.2</v>
+        <v>73</v>
       </c>
       <c r="D57" s="8" t="n">
         <v>21.9</v>
@@ -5032,395 +5032,395 @@
         <v>21.9</v>
       </c>
       <c r="F57" s="8" t="n">
-        <v>3.5</v>
+        <v>-9.4</v>
       </c>
       <c r="G57" s="9" t="n">
-        <v>79</v>
+        <v>68</v>
       </c>
       <c r="H57" s="10" t="n">
-        <v>8.4</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="58">
       <c r="A58" s="4" t="inlineStr">
         <is>
-          <t>2026-08-18</t>
+          <t>2026-08-19</t>
         </is>
       </c>
       <c r="B58" s="8" t="n">
-        <v>72.8</v>
+        <v>72.90000000000001</v>
       </c>
       <c r="C58" s="7" t="n">
-        <v>73</v>
+        <v>72.97</v>
       </c>
       <c r="D58" s="8" t="n">
-        <v>21.9</v>
+        <v>21.3</v>
       </c>
       <c r="E58" s="7" t="n">
-        <v>21.9</v>
+        <v>21.7</v>
       </c>
       <c r="F58" s="8" t="n">
-        <v>-9.4</v>
+        <v>-6.9</v>
       </c>
       <c r="G58" s="9" t="n">
-        <v>68</v>
+        <v>59</v>
       </c>
       <c r="H58" s="10" t="n">
-        <v>8.300000000000001</v>
+        <v>9.6</v>
       </c>
     </row>
     <row r="59">
       <c r="A59" s="4" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-20</t>
         </is>
       </c>
       <c r="B59" s="8" t="n">
-        <v>72.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C59" s="7" t="n">
-        <v>72.97</v>
+        <v>72.88</v>
       </c>
       <c r="D59" s="8" t="n">
-        <v>21.3</v>
+        <v>20.9</v>
       </c>
       <c r="E59" s="7" t="n">
-        <v>21.7</v>
+        <v>21.5</v>
       </c>
       <c r="F59" s="8" t="n">
-        <v>-6.9</v>
+        <v>-3.2</v>
       </c>
       <c r="G59" s="9" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H59" s="10" t="n">
-        <v>9.6</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="4" t="inlineStr">
         <is>
-          <t>2026-08-20</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B60" s="8" t="n">
-        <v>72.59999999999999</v>
+        <v>73.90000000000001</v>
       </c>
       <c r="C60" s="7" t="n">
-        <v>72.88</v>
+        <v>73.08</v>
       </c>
       <c r="D60" s="8" t="n">
         <v>20.9</v>
       </c>
       <c r="E60" s="7" t="n">
-        <v>21.5</v>
+        <v>21.38</v>
       </c>
       <c r="F60" s="8" t="n">
-        <v>-3.2</v>
+        <v>0.9</v>
       </c>
       <c r="G60" s="9" t="n">
-        <v>54</v>
+        <v>51</v>
       </c>
       <c r="H60" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>6.8</v>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="4" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-22</t>
         </is>
       </c>
       <c r="B61" s="8" t="n">
-        <v>73.90000000000001</v>
+        <v>72.59999999999999</v>
       </c>
       <c r="C61" s="7" t="n">
-        <v>73.08</v>
+        <v>73</v>
       </c>
       <c r="D61" s="8" t="n">
-        <v>20.9</v>
+        <v>21.8</v>
       </c>
       <c r="E61" s="7" t="n">
-        <v>21.38</v>
+        <v>21.45</v>
       </c>
       <c r="F61" s="8" t="n">
-        <v>0.9</v>
+        <v>2.7</v>
       </c>
       <c r="G61" s="9" t="n">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="H61" s="10" t="n">
-        <v>6.8</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="4" t="inlineStr">
         <is>
-          <t>2026-08-22</t>
-        </is>
-      </c>
-      <c r="B62" s="8" t="n">
-        <v>72.59999999999999</v>
-      </c>
+          <t>2026-08-23</t>
+        </is>
+      </c>
+      <c r="B62" s="8" t="n"/>
       <c r="C62" s="7" t="n">
         <v>73</v>
       </c>
-      <c r="D62" s="8" t="n">
-        <v>21.8</v>
-      </c>
+      <c r="D62" s="8" t="n"/>
       <c r="E62" s="7" t="n">
         <v>21.45</v>
       </c>
       <c r="F62" s="8" t="n">
-        <v>2.7</v>
+        <v>2.4</v>
       </c>
       <c r="G62" s="9" t="n">
-        <v>53</v>
+        <v>61</v>
       </c>
       <c r="H62" s="10" t="n">
-        <v>7.5</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="4" t="inlineStr">
         <is>
-          <t>2026-08-23</t>
-        </is>
-      </c>
-      <c r="B63" s="8" t="n"/>
+          <t>2026-08-24</t>
+        </is>
+      </c>
+      <c r="B63" s="8" t="n">
+        <v>71.90000000000001</v>
+      </c>
       <c r="C63" s="7" t="n">
-        <v>73</v>
-      </c>
-      <c r="D63" s="8" t="n"/>
+        <v>72.78</v>
+      </c>
+      <c r="D63" s="8" t="n">
+        <v>20.7</v>
+      </c>
       <c r="E63" s="7" t="n">
-        <v>21.45</v>
+        <v>21.25</v>
       </c>
       <c r="F63" s="8" t="n">
-        <v>2.4</v>
+        <v>4</v>
       </c>
       <c r="G63" s="9" t="n">
-        <v>61</v>
+        <v>59</v>
       </c>
       <c r="H63" s="10" t="n">
-        <v>7.7</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="4" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="B64" s="8" t="n">
-        <v>71.90000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="C64" s="7" t="n">
-        <v>72.78</v>
+        <v>72.56999999999999</v>
       </c>
       <c r="D64" s="8" t="n">
-        <v>20.7</v>
+        <v>21.6</v>
       </c>
       <c r="E64" s="7" t="n">
-        <v>21.25</v>
+        <v>21.2</v>
       </c>
       <c r="F64" s="8" t="n">
-        <v>4</v>
+        <v>-3.6</v>
       </c>
       <c r="G64" s="9" t="n">
-        <v>59</v>
+        <v>69</v>
       </c>
       <c r="H64" s="10" t="n">
-        <v>6.7</v>
+        <v>8.300000000000001</v>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="4" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="B65" s="8" t="n">
-        <v>71.5</v>
+        <v>71</v>
       </c>
       <c r="C65" s="7" t="n">
-        <v>72.56999999999999</v>
+        <v>72.25</v>
       </c>
       <c r="D65" s="8" t="n">
-        <v>21.6</v>
+        <v>21.9</v>
       </c>
       <c r="E65" s="7" t="n">
-        <v>21.2</v>
+        <v>21.3</v>
       </c>
       <c r="F65" s="8" t="n">
-        <v>-3.6</v>
+        <v>1</v>
       </c>
       <c r="G65" s="9" t="n">
-        <v>69</v>
+        <v>62</v>
       </c>
       <c r="H65" s="10" t="n">
-        <v>8.300000000000001</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="4" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-27</t>
         </is>
       </c>
       <c r="B66" s="8" t="n">
-        <v>71</v>
+        <v>71.59999999999999</v>
       </c>
       <c r="C66" s="7" t="n">
-        <v>72.25</v>
+        <v>72.08</v>
       </c>
       <c r="D66" s="8" t="n">
-        <v>21.9</v>
+        <v>21.4</v>
       </c>
       <c r="E66" s="7" t="n">
-        <v>21.3</v>
+        <v>21.38</v>
       </c>
       <c r="F66" s="8" t="n">
-        <v>1</v>
+        <v>5.9</v>
       </c>
       <c r="G66" s="9" t="n">
-        <v>62</v>
+        <v>49</v>
       </c>
       <c r="H66" s="10" t="n">
-        <v>8.4</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="4" t="inlineStr">
         <is>
-          <t>2026-08-27</t>
+          <t>2026-08-28</t>
         </is>
       </c>
       <c r="B67" s="8" t="n">
-        <v>71.59999999999999</v>
+        <v>72.3</v>
       </c>
       <c r="C67" s="7" t="n">
-        <v>72.08</v>
+        <v>71.81999999999999</v>
       </c>
       <c r="D67" s="8" t="n">
-        <v>21.4</v>
+        <v>20.8</v>
       </c>
       <c r="E67" s="7" t="n">
-        <v>21.38</v>
+        <v>21.37</v>
       </c>
       <c r="F67" s="8" t="n">
-        <v>5.9</v>
+        <v>9.5</v>
       </c>
       <c r="G67" s="9" t="n">
-        <v>49</v>
+        <v>80</v>
       </c>
       <c r="H67" s="10" t="n">
-        <v>8.6</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="4" t="inlineStr">
         <is>
-          <t>2026-08-28</t>
+          <t>2026-08-29</t>
         </is>
       </c>
       <c r="B68" s="8" t="n">
-        <v>72.3</v>
+        <v>72.5</v>
       </c>
       <c r="C68" s="7" t="n">
-        <v>71.81999999999999</v>
+        <v>71.8</v>
       </c>
       <c r="D68" s="8" t="n">
-        <v>20.8</v>
+        <v>21.6</v>
       </c>
       <c r="E68" s="7" t="n">
-        <v>21.37</v>
+        <v>21.33</v>
       </c>
       <c r="F68" s="8" t="n">
-        <v>9.5</v>
+        <v>6</v>
       </c>
       <c r="G68" s="9" t="n">
-        <v>80</v>
+        <v>49</v>
       </c>
       <c r="H68" s="10" t="n">
-        <v>8.4</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="4" t="inlineStr">
         <is>
-          <t>2026-08-29</t>
+          <t>2026-08-30</t>
         </is>
       </c>
       <c r="B69" s="8" t="n">
-        <v>72.5</v>
+        <v>73</v>
       </c>
       <c r="C69" s="7" t="n">
-        <v>71.8</v>
+        <v>71.97</v>
       </c>
       <c r="D69" s="8" t="n">
-        <v>21.6</v>
+        <v>22.1</v>
       </c>
       <c r="E69" s="7" t="n">
-        <v>21.33</v>
+        <v>21.44</v>
       </c>
       <c r="F69" s="8" t="n">
-        <v>6</v>
+        <v>2.7</v>
       </c>
       <c r="G69" s="9" t="n">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="H69" s="10" t="n">
-        <v>7.5</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="4" t="inlineStr">
         <is>
-          <t>2026-08-30</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="B70" s="8" t="n">
-        <v>73</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="C70" s="7" t="n">
-        <v>71.97</v>
+        <v>72.14</v>
       </c>
       <c r="D70" s="8" t="n">
-        <v>22.1</v>
+        <v>22.6</v>
       </c>
       <c r="E70" s="7" t="n">
-        <v>21.44</v>
+        <v>21.71</v>
       </c>
       <c r="F70" s="8" t="n">
-        <v>2.7</v>
+        <v>6.1</v>
       </c>
       <c r="G70" s="9" t="n">
-        <v>51</v>
+        <v>63</v>
       </c>
       <c r="H70" s="10" t="n">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="4" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-01</t>
         </is>
       </c>
       <c r="B71" s="8" t="n">
-        <v>73.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C71" s="7" t="n">
-        <v>72.14</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="D71" s="8" t="n">
-        <v>22.6</v>
+        <v>20.8</v>
       </c>
       <c r="E71" s="7" t="n">
-        <v>21.71</v>
+        <v>21.6</v>
       </c>
       <c r="F71" s="8" t="n">
-        <v>6.1</v>
+        <v>4.8</v>
       </c>
       <c r="G71" s="9" t="n">
         <v>63</v>
@@ -5432,187 +5432,183 @@
     <row r="72">
       <c r="A72" s="4" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="B72" s="8" t="n">
-        <v>72.2</v>
+        <v>72.3</v>
       </c>
       <c r="C72" s="7" t="n">
-        <v>72.23999999999999</v>
+        <v>72.43000000000001</v>
       </c>
       <c r="D72" s="8" t="n">
-        <v>20.8</v>
+        <v>21.3</v>
       </c>
       <c r="E72" s="7" t="n">
-        <v>21.6</v>
+        <v>21.51</v>
       </c>
       <c r="F72" s="8" t="n">
-        <v>4.8</v>
+        <v>5</v>
       </c>
       <c r="G72" s="9" t="n">
-        <v>63</v>
+        <v>72</v>
       </c>
       <c r="H72" s="10" t="n">
-        <v>7.7</v>
+        <v>7.8</v>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="4" t="inlineStr">
         <is>
-          <t>2026-09-02</t>
+          <t>2026-09-03</t>
         </is>
       </c>
       <c r="B73" s="8" t="n">
         <v>72.3</v>
       </c>
       <c r="C73" s="7" t="n">
-        <v>72.43000000000001</v>
+        <v>72.53</v>
       </c>
       <c r="D73" s="8" t="n">
-        <v>21.3</v>
+        <v>21.9</v>
       </c>
       <c r="E73" s="7" t="n">
-        <v>21.51</v>
+        <v>21.59</v>
       </c>
       <c r="F73" s="8" t="n">
-        <v>5</v>
+        <v>5.3</v>
       </c>
       <c r="G73" s="9" t="n">
-        <v>72</v>
+        <v>48</v>
       </c>
       <c r="H73" s="10" t="n">
-        <v>7.8</v>
+        <v>8.9</v>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="4" t="inlineStr">
         <is>
-          <t>2026-09-03</t>
-        </is>
-      </c>
-      <c r="B74" s="8" t="n">
-        <v>72.3</v>
-      </c>
+          <t>2026-09-04</t>
+        </is>
+      </c>
+      <c r="B74" s="8" t="n"/>
       <c r="C74" s="7" t="n">
-        <v>72.53</v>
-      </c>
-      <c r="D74" s="8" t="n">
-        <v>21.9</v>
-      </c>
+        <v>72.56999999999999</v>
+      </c>
+      <c r="D74" s="8" t="n"/>
       <c r="E74" s="7" t="n">
-        <v>21.59</v>
+        <v>21.72</v>
       </c>
       <c r="F74" s="8" t="n">
-        <v>5.3</v>
+        <v>7.7</v>
       </c>
       <c r="G74" s="9" t="n">
-        <v>48</v>
+        <v>59</v>
       </c>
       <c r="H74" s="10" t="n">
-        <v>8.9</v>
+        <v>6.6</v>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="4" t="inlineStr">
         <is>
-          <t>2026-09-04</t>
+          <t>2026-09-05</t>
         </is>
       </c>
       <c r="B75" s="8" t="n"/>
       <c r="C75" s="7" t="n">
-        <v>72.56999999999999</v>
+        <v>72.58</v>
       </c>
       <c r="D75" s="8" t="n"/>
       <c r="E75" s="7" t="n">
-        <v>21.72</v>
+        <v>21.74</v>
       </c>
       <c r="F75" s="8" t="n">
-        <v>7.7</v>
+        <v>-7.3</v>
       </c>
       <c r="G75" s="9" t="n">
-        <v>59</v>
+        <v>54</v>
       </c>
       <c r="H75" s="10" t="n">
-        <v>6.6</v>
+        <v>4.1</v>
       </c>
     </row>
     <row r="76">
       <c r="A76" s="4" t="inlineStr">
         <is>
-          <t>2026-09-05</t>
+          <t>2026-09-06</t>
         </is>
       </c>
       <c r="B76" s="8" t="n"/>
       <c r="C76" s="7" t="n">
-        <v>72.58</v>
+        <v>72.48</v>
       </c>
       <c r="D76" s="8" t="n"/>
       <c r="E76" s="7" t="n">
-        <v>21.74</v>
+        <v>21.65</v>
       </c>
       <c r="F76" s="8" t="n">
-        <v>-7.3</v>
+        <v>-2.2</v>
       </c>
       <c r="G76" s="9" t="n">
-        <v>54</v>
+        <v>35</v>
       </c>
       <c r="H76" s="10" t="n">
-        <v>4.1</v>
+        <v>8</v>
       </c>
     </row>
     <row r="77">
       <c r="A77" s="4" t="inlineStr">
         <is>
-          <t>2026-09-06</t>
+          <t>2026-09-07</t>
         </is>
       </c>
       <c r="B77" s="8" t="n"/>
       <c r="C77" s="7" t="n">
-        <v>72.48</v>
+        <v>72.27</v>
       </c>
       <c r="D77" s="8" t="n"/>
       <c r="E77" s="7" t="n">
-        <v>21.65</v>
+        <v>21.33</v>
       </c>
       <c r="F77" s="8" t="n">
-        <v>-2.2</v>
+        <v>1.7</v>
       </c>
       <c r="G77" s="9" t="n">
-        <v>35</v>
+        <v>50</v>
       </c>
       <c r="H77" s="10" t="n">
-        <v>8</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="78">
       <c r="A78" s="4" t="inlineStr">
         <is>
-          <t>2026-09-07</t>
+          <t>2026-09-08</t>
         </is>
       </c>
       <c r="B78" s="8" t="n"/>
       <c r="C78" s="7" t="n">
-        <v>72.27</v>
+        <v>72.3</v>
       </c>
       <c r="D78" s="8" t="n"/>
       <c r="E78" s="7" t="n">
-        <v>21.33</v>
+        <v>21.6</v>
       </c>
       <c r="F78" s="8" t="n">
-        <v>1.7</v>
+        <v>5</v>
       </c>
       <c r="G78" s="9" t="n">
-        <v>50</v>
+        <v>65</v>
       </c>
       <c r="H78" s="10" t="n">
-        <v>7.7</v>
+        <v>7.6</v>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="4" t="inlineStr">
         <is>
-          <t>2026-09-08</t>
+          <t>2026-09-09</t>
         </is>
       </c>
       <c r="B79" s="8" t="n"/>
@@ -5621,433 +5617,429 @@
       </c>
       <c r="D79" s="8" t="n"/>
       <c r="E79" s="7" t="n">
-        <v>21.6</v>
+        <v>21.9</v>
       </c>
       <c r="F79" s="8" t="n">
-        <v>5</v>
+        <v>1.9</v>
       </c>
       <c r="G79" s="9" t="n">
-        <v>65</v>
+        <v>54</v>
       </c>
       <c r="H79" s="10" t="n">
-        <v>7.6</v>
+        <v>7.5</v>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="4" t="inlineStr">
         <is>
-          <t>2026-09-09</t>
-        </is>
-      </c>
-      <c r="B80" s="8" t="n"/>
+          <t>2026-09-10</t>
+        </is>
+      </c>
+      <c r="B80" s="8" t="n">
+        <v>73.7</v>
+      </c>
       <c r="C80" s="7" t="n">
-        <v>72.3</v>
-      </c>
-      <c r="D80" s="8" t="n"/>
+        <v>73.7</v>
+      </c>
+      <c r="D80" s="8" t="n">
+        <v>20.9</v>
+      </c>
       <c r="E80" s="7" t="n">
-        <v>21.9</v>
+        <v>20.9</v>
       </c>
       <c r="F80" s="8" t="n">
-        <v>1.9</v>
+        <v>2.2</v>
       </c>
       <c r="G80" s="9" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H80" s="10" t="n">
-        <v>7.5</v>
+        <v>6.7</v>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="4" t="inlineStr">
         <is>
-          <t>2026-09-10</t>
+          <t>2026-09-11</t>
         </is>
       </c>
       <c r="B81" s="8" t="n">
-        <v>73.7</v>
+        <v>72.5</v>
       </c>
       <c r="C81" s="7" t="n">
-        <v>73.7</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="D81" s="8" t="n">
-        <v>20.9</v>
+        <v>21.4</v>
       </c>
       <c r="E81" s="7" t="n">
-        <v>20.9</v>
+        <v>21.15</v>
       </c>
       <c r="F81" s="8" t="n">
-        <v>2.2</v>
+        <v>5.9</v>
       </c>
       <c r="G81" s="9" t="n">
-        <v>66</v>
+        <v>59</v>
       </c>
       <c r="H81" s="10" t="n">
-        <v>6.7</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="4" t="inlineStr">
         <is>
-          <t>2026-09-11</t>
+          <t>2026-09-12</t>
         </is>
       </c>
       <c r="B82" s="8" t="n">
-        <v>72.5</v>
+        <v>72.3</v>
       </c>
       <c r="C82" s="7" t="n">
-        <v>73.09999999999999</v>
+        <v>72.83</v>
       </c>
       <c r="D82" s="8" t="n">
+        <v>21.9</v>
+      </c>
+      <c r="E82" s="7" t="n">
         <v>21.4</v>
       </c>
-      <c r="E82" s="7" t="n">
-        <v>21.15</v>
-      </c>
       <c r="F82" s="8" t="n">
-        <v>5.9</v>
+        <v>4</v>
       </c>
       <c r="G82" s="9" t="n">
-        <v>59</v>
+        <v>57</v>
       </c>
       <c r="H82" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>9.5</v>
       </c>
     </row>
     <row r="83">
       <c r="A83" s="4" t="inlineStr">
         <is>
-          <t>2026-09-12</t>
+          <t>2026-09-13</t>
         </is>
       </c>
       <c r="B83" s="8" t="n">
-        <v>72.3</v>
+        <v>71.8</v>
       </c>
       <c r="C83" s="7" t="n">
-        <v>72.83</v>
+        <v>72.58</v>
       </c>
       <c r="D83" s="8" t="n">
-        <v>21.9</v>
+        <v>22.4</v>
       </c>
       <c r="E83" s="7" t="n">
-        <v>21.4</v>
+        <v>21.65</v>
       </c>
       <c r="F83" s="8" t="n">
-        <v>4</v>
+        <v>1.4</v>
       </c>
       <c r="G83" s="9" t="n">
-        <v>57</v>
+        <v>45</v>
       </c>
       <c r="H83" s="10" t="n">
-        <v>9.5</v>
+        <v>9.699999999999999</v>
       </c>
     </row>
     <row r="84">
       <c r="A84" s="4" t="inlineStr">
         <is>
-          <t>2026-09-13</t>
+          <t>2026-09-14</t>
         </is>
       </c>
       <c r="B84" s="8" t="n">
-        <v>71.8</v>
+        <v>70.90000000000001</v>
       </c>
       <c r="C84" s="7" t="n">
-        <v>72.58</v>
+        <v>72.23999999999999</v>
       </c>
       <c r="D84" s="8" t="n">
-        <v>22.4</v>
+        <v>20.9</v>
       </c>
       <c r="E84" s="7" t="n">
-        <v>21.65</v>
+        <v>21.5</v>
       </c>
       <c r="F84" s="8" t="n">
-        <v>1.4</v>
+        <v>-0</v>
       </c>
       <c r="G84" s="9" t="n">
-        <v>45</v>
+        <v>58</v>
       </c>
       <c r="H84" s="10" t="n">
-        <v>9.699999999999999</v>
+        <v>8</v>
       </c>
     </row>
     <row r="85">
       <c r="A85" s="4" t="inlineStr">
         <is>
-          <t>2026-09-14</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="B85" s="8" t="n">
-        <v>70.90000000000001</v>
+        <v>71.7</v>
       </c>
       <c r="C85" s="7" t="n">
-        <v>72.23999999999999</v>
+        <v>72.15000000000001</v>
       </c>
       <c r="D85" s="8" t="n">
-        <v>20.9</v>
+        <v>21.6</v>
       </c>
       <c r="E85" s="7" t="n">
-        <v>21.5</v>
+        <v>21.52</v>
       </c>
       <c r="F85" s="8" t="n">
-        <v>-0</v>
+        <v>-0.9</v>
       </c>
       <c r="G85" s="9" t="n">
-        <v>58</v>
+        <v>54</v>
       </c>
       <c r="H85" s="10" t="n">
-        <v>8</v>
+        <v>7.1</v>
       </c>
     </row>
     <row r="86">
       <c r="A86" s="4" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-09-16</t>
         </is>
       </c>
       <c r="B86" s="8" t="n">
-        <v>71.7</v>
+        <v>71.40000000000001</v>
       </c>
       <c r="C86" s="7" t="n">
-        <v>72.15000000000001</v>
+        <v>72.04000000000001</v>
       </c>
       <c r="D86" s="8" t="n">
-        <v>21.6</v>
+        <v>21.5</v>
       </c>
       <c r="E86" s="7" t="n">
-        <v>21.52</v>
+        <v>21.51</v>
       </c>
       <c r="F86" s="8" t="n">
-        <v>-0.9</v>
+        <v>0.8</v>
       </c>
       <c r="G86" s="9" t="n">
-        <v>54</v>
+        <v>66</v>
       </c>
       <c r="H86" s="10" t="n">
-        <v>7.1</v>
+        <v>8.199999999999999</v>
       </c>
     </row>
     <row r="87">
       <c r="A87" s="4" t="inlineStr">
         <is>
-          <t>2026-09-16</t>
+          <t>2026-09-17</t>
         </is>
       </c>
       <c r="B87" s="8" t="n">
-        <v>71.40000000000001</v>
+        <v>71.5</v>
       </c>
       <c r="C87" s="7" t="n">
-        <v>72.04000000000001</v>
+        <v>71.73</v>
       </c>
       <c r="D87" s="8" t="n">
-        <v>21.5</v>
+        <v>21.6</v>
       </c>
       <c r="E87" s="7" t="n">
-        <v>21.51</v>
+        <v>21.61</v>
       </c>
       <c r="F87" s="8" t="n">
-        <v>0.8</v>
+        <v>0.4</v>
       </c>
       <c r="G87" s="9" t="n">
-        <v>66</v>
+        <v>55</v>
       </c>
       <c r="H87" s="10" t="n">
-        <v>8.199999999999999</v>
+        <v>8.4</v>
       </c>
     </row>
     <row r="88">
       <c r="A88" s="4" t="inlineStr">
         <is>
-          <t>2026-09-17</t>
+          <t>2026-09-18</t>
         </is>
       </c>
       <c r="B88" s="8" t="n">
-        <v>71.5</v>
+        <v>72.3</v>
       </c>
       <c r="C88" s="7" t="n">
-        <v>71.73</v>
+        <v>71.7</v>
       </c>
       <c r="D88" s="8" t="n">
+        <v>21.3</v>
+      </c>
+      <c r="E88" s="7" t="n">
         <v>21.6</v>
       </c>
-      <c r="E88" s="7" t="n">
-        <v>21.61</v>
-      </c>
       <c r="F88" s="8" t="n">
-        <v>0.4</v>
+        <v>5</v>
       </c>
       <c r="G88" s="9" t="n">
-        <v>55</v>
+        <v>59</v>
       </c>
       <c r="H88" s="10" t="n">
-        <v>8.4</v>
+        <v>8</v>
       </c>
     </row>
     <row r="89">
       <c r="A89" s="4" t="inlineStr">
         <is>
-          <t>2026-09-18</t>
+          <t>2026-09-19</t>
         </is>
       </c>
       <c r="B89" s="8" t="n">
-        <v>72.3</v>
+        <v>72.5</v>
       </c>
       <c r="C89" s="7" t="n">
-        <v>71.7</v>
+        <v>71.73</v>
       </c>
       <c r="D89" s="8" t="n">
-        <v>21.3</v>
+        <v>21.1</v>
       </c>
       <c r="E89" s="7" t="n">
-        <v>21.6</v>
+        <v>21.49</v>
       </c>
       <c r="F89" s="8" t="n">
-        <v>5</v>
+        <v>8.1</v>
       </c>
       <c r="G89" s="9" t="n">
-        <v>59</v>
+        <v>31</v>
       </c>
       <c r="H89" s="10" t="n">
-        <v>8</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="90">
       <c r="A90" s="4" t="inlineStr">
         <is>
-          <t>2026-09-19</t>
+          <t>2026-09-20</t>
         </is>
       </c>
       <c r="B90" s="8" t="n">
-        <v>72.5</v>
+        <v>73.3</v>
       </c>
       <c r="C90" s="7" t="n">
-        <v>71.73</v>
+        <v>71.94</v>
       </c>
       <c r="D90" s="8" t="n">
-        <v>21.1</v>
+        <v>22.2</v>
       </c>
       <c r="E90" s="7" t="n">
-        <v>21.49</v>
+        <v>21.46</v>
       </c>
       <c r="F90" s="8" t="n">
-        <v>8.1</v>
+        <v>-7.5</v>
       </c>
       <c r="G90" s="9" t="n">
-        <v>31</v>
+        <v>49</v>
       </c>
       <c r="H90" s="10" t="n">
-        <v>8.1</v>
+        <v>7.2</v>
       </c>
     </row>
     <row r="91">
       <c r="A91" s="4" t="inlineStr">
         <is>
-          <t>2026-09-20</t>
+          <t>2026-09-21</t>
         </is>
       </c>
       <c r="B91" s="8" t="n">
-        <v>73.3</v>
+        <v>73.2</v>
       </c>
       <c r="C91" s="7" t="n">
-        <v>71.94</v>
+        <v>72.27</v>
       </c>
       <c r="D91" s="8" t="n">
         <v>22.2</v>
       </c>
       <c r="E91" s="7" t="n">
-        <v>21.46</v>
+        <v>21.64</v>
       </c>
       <c r="F91" s="8" t="n">
-        <v>-7.5</v>
+        <v>-3.3</v>
       </c>
       <c r="G91" s="9" t="n">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="H91" s="10" t="n">
-        <v>7.2</v>
+        <v>8.6</v>
       </c>
     </row>
     <row r="92">
       <c r="A92" s="4" t="inlineStr">
         <is>
-          <t>2026-09-21</t>
+          <t>2026-09-22</t>
         </is>
       </c>
       <c r="B92" s="8" t="n">
-        <v>73.2</v>
+        <v>73.09999999999999</v>
       </c>
       <c r="C92" s="7" t="n">
-        <v>72.27</v>
+        <v>72.47</v>
       </c>
       <c r="D92" s="8" t="n">
-        <v>22.2</v>
+        <v>20.9</v>
       </c>
       <c r="E92" s="7" t="n">
-        <v>21.64</v>
+        <v>21.54</v>
       </c>
       <c r="F92" s="8" t="n">
-        <v>-3.3</v>
+        <v>1.2</v>
       </c>
       <c r="G92" s="9" t="n">
-        <v>45</v>
+        <v>51</v>
       </c>
       <c r="H92" s="10" t="n">
-        <v>8.6</v>
+        <v>7.7</v>
       </c>
     </row>
     <row r="93">
       <c r="A93" s="4" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-09-23</t>
         </is>
       </c>
       <c r="B93" s="8" t="n">
-        <v>73.09999999999999</v>
+        <v>72.2</v>
       </c>
       <c r="C93" s="7" t="n">
-        <v>72.47</v>
+        <v>72.59</v>
       </c>
       <c r="D93" s="8" t="n">
-        <v>20.9</v>
+        <v>21.1</v>
       </c>
       <c r="E93" s="7" t="n">
-        <v>21.54</v>
+        <v>21.49</v>
       </c>
       <c r="F93" s="8" t="n">
-        <v>1.2</v>
+        <v>-0.6</v>
       </c>
       <c r="G93" s="9" t="n">
-        <v>51</v>
+        <v>58</v>
       </c>
       <c r="H93" s="10" t="n">
-        <v>7.7</v>
+        <v>8.1</v>
       </c>
     </row>
     <row r="94">
       <c r="A94" s="4" t="inlineStr">
         <is>
-          <t>2026-09-23</t>
-        </is>
-      </c>
-      <c r="B94" s="8" t="n">
-        <v>72.2</v>
-      </c>
+          <t>2026-09-24</t>
+        </is>
+      </c>
+      <c r="B94" s="8" t="n"/>
       <c r="C94" s="7" t="n">
-        <v>72.59</v>
-      </c>
-      <c r="D94" s="8" t="n">
-        <v>21.1</v>
-      </c>
+        <v>72.77</v>
+      </c>
+      <c r="D94" s="8" t="n"/>
       <c r="E94" s="7" t="n">
-        <v>21.49</v>
+        <v>21.47</v>
       </c>
       <c r="F94" s="8" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="G94" s="9" t="n">
-        <v>58</v>
-      </c>
-      <c r="H94" s="10" t="n">
-        <v>8.1</v>
-      </c>
+        <v>-0.7</v>
+      </c>
+      <c r="G94" s="9" t="n"/>
+      <c r="H94" s="10" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6207,16 +6199,16 @@
         <v>53</v>
       </c>
       <c r="E7" s="8" t="n">
-        <v>48.5</v>
+        <v>48.7</v>
       </c>
       <c r="F7" s="4" t="n">
         <v>415</v>
       </c>
       <c r="G7" s="4" t="n">
-        <v>33</v>
+        <v>41</v>
       </c>
       <c r="H7" s="11" t="n">
-        <v>-382</v>
+        <v>-374</v>
       </c>
     </row>
     <row r="8">

</xml_diff>